<commit_message>
Use the employer share of the Spanish solidarity contribution (0.96%)
The rate above the contribution ceiling was 1.15%, which is the combined
employer + worker rate of the first band of the cuota de solidaridad
(2026). The models count employer cost, so the default is now the
employer share, 0.96%. Totals move by a few hundred euros; the
calculator, the payroll budget dashboard and both Excel models are
rebuilt and recalculated, and all checks pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/budget-plan-fact/budget-plan-fact-model.xlsx
+++ b/budget-plan-fact/budget-plan-fact-model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Projects IA\PROJECT-pay-gap-calculator\budget-plan-fact\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2DC47A0-7C92-4DA1-85D3-D54E27FB4DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03EA00B2-26DA-4133-9123-3DDA0A1C0948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -494,7 +494,7 @@
     <t>Employer contributions</t>
   </si>
   <si>
-    <t>A raise to base pay brings employer contributions with it, and those are part of the budget line. The rates here are Spain 2026: 31.5% on annual pay up to a ceiling of 61,214 EUR, and 1.15% on anything above it. The scale is regressive, so a raise to someone already above the ceiling attracts almost no contributions while the same raise below it attracts the full rate. That is why the effective rate on the Equalisation sheet differs so much between departments. Rates and ceiling are specific to one country and one year: in another jurisdiction the numbers change, the structure does not.</t>
+    <t>A raise to base pay brings employer contributions with it, and those are part of the budget line. The rates here are Spain 2026: 31.5% on annual pay up to a ceiling of 61,214 EUR, and 0.96% on anything above it (the employer share of the first band of the solidarity contribution, 0.96% of the combined 1.15%). The scale is regressive, so a raise to someone already above the ceiling attracts almost no contributions while the same raise below it attracts the full rate. That is why the effective rate on the Equalisation sheet differs so much between departments. Rates and ceiling are specific to one country and one year: in another jurisdiction the numbers change, the structure does not.</t>
   </si>
   <si>
     <t>Synthetic data</t>
@@ -1118,15 +1118,15 @@
         <v>77733.194175898621</v>
       </c>
       <c r="D8" s="9">
-        <v>20286.974469272041</v>
+        <v>20260.68759868668</v>
       </c>
       <c r="E8" s="10">
         <f t="shared" ref="E8:E14" si="0">C8+D8</f>
-        <v>98020.168645170663</v>
+        <v>97993.881774585301</v>
       </c>
       <c r="F8" s="10">
         <f t="shared" ref="F8:F14" si="1">E8/12</f>
-        <v>8168.3473870975549</v>
+        <v>8166.1568145487754</v>
       </c>
       <c r="G8" s="11">
         <v>-1.4409976867000001</v>
@@ -1143,15 +1143,15 @@
         <v>124991.43000000009</v>
       </c>
       <c r="D9" s="9">
-        <v>4866.7996950000024</v>
+        <v>4650.7850279999993</v>
       </c>
       <c r="E9" s="10">
         <f t="shared" si="0"/>
-        <v>129858.2296950001</v>
+        <v>129642.21502800009</v>
       </c>
       <c r="F9" s="10">
         <f t="shared" si="1"/>
-        <v>10821.519141250008</v>
+        <v>10803.517919000007</v>
       </c>
       <c r="G9" s="11">
         <v>9.2535006260999992</v>
@@ -1268,15 +1268,15 @@
         <v>18287.125943342169</v>
       </c>
       <c r="D14" s="9">
-        <v>210.30194834843499</v>
+        <v>175.55640905608479</v>
       </c>
       <c r="E14" s="10">
         <f t="shared" si="0"/>
-        <v>18497.427891690604</v>
+        <v>18462.682352398253</v>
       </c>
       <c r="F14" s="10">
         <f t="shared" si="1"/>
-        <v>1541.4523243075503</v>
+        <v>1538.5568626998545</v>
       </c>
       <c r="G14" s="11">
         <v>2.6526177826000001</v>
@@ -1296,15 +1296,15 @@
       </c>
       <c r="D15" s="13">
         <f>SUM(D8:D14)</f>
-        <v>61330.546831881788</v>
+        <v>61053.499755004072</v>
       </c>
       <c r="E15" s="13">
         <f>SUM(E8:E14)</f>
-        <v>396521.56907576183</v>
+        <v>396244.5219988841</v>
       </c>
       <c r="F15" s="13">
         <f>SUM(F8:F14)</f>
-        <v>33043.464089646812</v>
+        <v>33020.376833240334</v>
       </c>
     </row>
   </sheetData>
@@ -1382,10 +1382,10 @@
         <v>1</v>
       </c>
       <c r="D5" s="9">
-        <v>344874.17</v>
+        <v>344781.5</v>
       </c>
       <c r="E5" s="9">
-        <v>339482.19</v>
+        <v>339390.97</v>
       </c>
       <c r="F5" s="10" t="str">
         <f>IF(C5&lt;=fact_months,"",ROUND(D5*(1+Equalisation!$G$8/100)+IF(C5&gt;=equalisation_month,Equalisation!$F$8,0),2))</f>
@@ -1393,19 +1393,19 @@
       </c>
       <c r="G5" s="10">
         <f t="shared" ref="G5:G36" si="0">IF(C5&lt;=fact_months,E5,F5)</f>
-        <v>339482.19</v>
+        <v>339390.97</v>
       </c>
       <c r="H5" s="10">
         <f t="shared" ref="H5:H36" si="1">G5-D5</f>
-        <v>-5391.9799999999814</v>
+        <v>-5390.5300000000279</v>
       </c>
       <c r="I5" s="14">
         <f t="shared" ref="I5:I36" si="2">IF(D5=0,"",H5/D5)</f>
-        <v>-1.5634629870946791E-2</v>
+        <v>-1.5634626567840874E-2</v>
       </c>
       <c r="J5" s="10">
         <f>H5</f>
-        <v>-5391.9799999999814</v>
+        <v>-5390.5300000000279</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -1419,10 +1419,10 @@
         <v>2</v>
       </c>
       <c r="D6" s="9">
-        <v>343877.42</v>
+        <v>343785.02</v>
       </c>
       <c r="E6" s="9">
-        <v>338599.58</v>
+        <v>338508.59</v>
       </c>
       <c r="F6" s="10" t="str">
         <f>IF(C6&lt;=fact_months,"",ROUND(D6*(1+Equalisation!$G$8/100)+IF(C6&gt;=equalisation_month,Equalisation!$F$8,0),2))</f>
@@ -1430,19 +1430,19 @@
       </c>
       <c r="G6" s="10">
         <f t="shared" si="0"/>
-        <v>338599.58</v>
+        <v>338508.59</v>
       </c>
       <c r="H6" s="10">
         <f t="shared" si="1"/>
-        <v>-5277.8399999999674</v>
+        <v>-5276.429999999993</v>
       </c>
       <c r="I6" s="14">
         <f t="shared" si="2"/>
-        <v>-1.5348027212720066E-2</v>
+        <v>-1.5348050941835665E-2</v>
       </c>
       <c r="J6" s="10">
         <f t="shared" ref="J6:J16" si="3">J5+H6</f>
-        <v>-10669.819999999949</v>
+        <v>-10666.960000000021</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
@@ -1456,10 +1456,10 @@
         <v>3</v>
       </c>
       <c r="D7" s="9">
-        <v>339558.19</v>
+        <v>339466.94</v>
       </c>
       <c r="E7" s="9">
-        <v>334287.48</v>
+        <v>334197.65000000002</v>
       </c>
       <c r="F7" s="10" t="str">
         <f>IF(C7&lt;=fact_months,"",ROUND(D7*(1+Equalisation!$G$8/100)+IF(C7&gt;=equalisation_month,Equalisation!$F$8,0),2))</f>
@@ -1467,19 +1467,19 @@
       </c>
       <c r="G7" s="10">
         <f t="shared" si="0"/>
-        <v>334287.48</v>
+        <v>334197.65000000002</v>
       </c>
       <c r="H7" s="10">
         <f t="shared" si="1"/>
-        <v>-5270.710000000021</v>
+        <v>-5269.289999999979</v>
       </c>
       <c r="I7" s="14">
         <f t="shared" si="2"/>
-        <v>-1.5522258497137179E-2</v>
+        <v>-1.5522247910208809E-2</v>
       </c>
       <c r="J7" s="10">
         <f t="shared" si="3"/>
-        <v>-15940.52999999997</v>
+        <v>-15936.25</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
@@ -1493,10 +1493,10 @@
         <v>4</v>
       </c>
       <c r="D8" s="9">
-        <v>333909.96000000002</v>
+        <v>333820.23</v>
       </c>
       <c r="E8" s="9">
-        <v>329292.71000000002</v>
+        <v>329204.23</v>
       </c>
       <c r="F8" s="10" t="str">
         <f>IF(C8&lt;=fact_months,"",ROUND(D8*(1+Equalisation!$G$8/100)+IF(C8&gt;=equalisation_month,Equalisation!$F$8,0),2))</f>
@@ -1504,19 +1504,19 @@
       </c>
       <c r="G8" s="10">
         <f t="shared" si="0"/>
-        <v>329292.71000000002</v>
+        <v>329204.23</v>
       </c>
       <c r="H8" s="10">
         <f t="shared" si="1"/>
-        <v>-4617.25</v>
+        <v>-4616</v>
       </c>
       <c r="I8" s="14">
         <f t="shared" si="2"/>
-        <v>-1.3827829514279837E-2</v>
+        <v>-1.3827801868089301E-2</v>
       </c>
       <c r="J8" s="10">
         <f t="shared" si="3"/>
-        <v>-20557.77999999997</v>
+        <v>-20552.25</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -1530,10 +1530,10 @@
         <v>5</v>
       </c>
       <c r="D9" s="9">
-        <v>327597.23</v>
+        <v>327509.2</v>
       </c>
       <c r="E9" s="9">
-        <v>323163.59999999998</v>
+        <v>323076.76</v>
       </c>
       <c r="F9" s="10" t="str">
         <f>IF(C9&lt;=fact_months,"",ROUND(D9*(1+Equalisation!$G$8/100)+IF(C9&gt;=equalisation_month,Equalisation!$F$8,0),2))</f>
@@ -1541,19 +1541,19 @@
       </c>
       <c r="G9" s="10">
         <f t="shared" si="0"/>
-        <v>323163.59999999998</v>
+        <v>323076.76</v>
       </c>
       <c r="H9" s="10">
         <f t="shared" si="1"/>
-        <v>-4433.6300000000047</v>
+        <v>-4432.4400000000023</v>
       </c>
       <c r="I9" s="14">
         <f t="shared" si="2"/>
-        <v>-1.3533783542675268E-2</v>
+        <v>-1.3533787753137934E-2</v>
       </c>
       <c r="J9" s="10">
         <f t="shared" si="3"/>
-        <v>-24991.409999999974</v>
+        <v>-24984.690000000002</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
@@ -1567,10 +1567,10 @@
         <v>6</v>
       </c>
       <c r="D10" s="9">
-        <v>321616.76</v>
+        <v>321530.33</v>
       </c>
       <c r="E10" s="9">
-        <v>316851.64</v>
+        <v>316766.49</v>
       </c>
       <c r="F10" s="10" t="str">
         <f>IF(C10&lt;=fact_months,"",ROUND(D10*(1+Equalisation!$G$8/100)+IF(C10&gt;=equalisation_month,Equalisation!$F$8,0),2))</f>
@@ -1578,19 +1578,19 @@
       </c>
       <c r="G10" s="10">
         <f t="shared" si="0"/>
-        <v>316851.64</v>
+        <v>316766.49</v>
       </c>
       <c r="H10" s="10">
         <f t="shared" si="1"/>
-        <v>-4765.1199999999953</v>
+        <v>-4763.8400000000256</v>
       </c>
       <c r="I10" s="14">
         <f t="shared" si="2"/>
-        <v>-1.4816143288054999E-2</v>
+        <v>-1.4816145027438081E-2</v>
       </c>
       <c r="J10" s="10">
         <f t="shared" si="3"/>
-        <v>-29756.52999999997</v>
+        <v>-29748.530000000028</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
@@ -1604,10 +1604,10 @@
         <v>7</v>
       </c>
       <c r="D11" s="9">
-        <v>319623.26</v>
+        <v>319537.38</v>
       </c>
       <c r="E11" s="9">
-        <v>314626.40000000002</v>
+        <v>314541.87</v>
       </c>
       <c r="F11" s="10" t="str">
         <f>IF(C11&lt;=fact_months,"",ROUND(D11*(1+Equalisation!$G$8/100)+IF(C11&gt;=equalisation_month,Equalisation!$F$8,0),2))</f>
@@ -1615,19 +1615,19 @@
       </c>
       <c r="G11" s="10">
         <f t="shared" si="0"/>
-        <v>314626.40000000002</v>
+        <v>314541.87</v>
       </c>
       <c r="H11" s="10">
         <f t="shared" si="1"/>
-        <v>-4996.859999999986</v>
+        <v>-4995.5100000000093</v>
       </c>
       <c r="I11" s="14">
         <f t="shared" si="2"/>
-        <v>-1.5633593124605469E-2</v>
+        <v>-1.5633570006739147E-2</v>
       </c>
       <c r="J11" s="10">
         <f t="shared" si="3"/>
-        <v>-34753.389999999956</v>
+        <v>-34744.040000000037</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
@@ -1641,10 +1641,10 @@
         <v>8</v>
       </c>
       <c r="D12" s="9">
-        <v>320287.76</v>
+        <v>320201.7</v>
       </c>
       <c r="E12" s="9">
-        <v>315905.42</v>
+        <v>315820.53000000003</v>
       </c>
       <c r="F12" s="10" t="str">
         <f>IF(C12&lt;=fact_months,"",ROUND(D12*(1+Equalisation!$G$8/100)+IF(C12&gt;=equalisation_month,Equalisation!$F$8,0),2))</f>
@@ -1652,19 +1652,19 @@
       </c>
       <c r="G12" s="10">
         <f t="shared" si="0"/>
-        <v>315905.42</v>
+        <v>315820.53000000003</v>
       </c>
       <c r="H12" s="10">
         <f t="shared" si="1"/>
-        <v>-4382.3400000000256</v>
+        <v>-4381.1699999999837</v>
       </c>
       <c r="I12" s="14">
         <f t="shared" si="2"/>
-        <v>-1.3682508504227652E-2</v>
+        <v>-1.3682531979061895E-2</v>
       </c>
       <c r="J12" s="10">
         <f t="shared" si="3"/>
-        <v>-39135.729999999981</v>
+        <v>-39125.210000000021</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
@@ -1678,28 +1678,28 @@
         <v>9</v>
       </c>
       <c r="D13" s="9">
-        <v>327264.98</v>
+        <v>327177.05</v>
       </c>
       <c r="E13" s="4"/>
       <c r="F13" s="10">
         <f>IF(C13&lt;=fact_months,"",ROUND(D13*(1+Equalisation!$G$8/100)+IF(C13&gt;=equalisation_month,Equalisation!$F$8,0),2))</f>
-        <v>330717.45</v>
+        <v>330628.59000000003</v>
       </c>
       <c r="G13" s="10">
         <f t="shared" si="0"/>
-        <v>330717.45</v>
+        <v>330628.59000000003</v>
       </c>
       <c r="H13" s="10">
         <f t="shared" si="1"/>
-        <v>3452.4700000000303</v>
+        <v>3451.5400000000373</v>
       </c>
       <c r="I13" s="14">
         <f t="shared" si="2"/>
-        <v>1.0549463618136076E-2</v>
+        <v>1.0549456326475337E-2</v>
       </c>
       <c r="J13" s="10">
         <f t="shared" si="3"/>
-        <v>-35683.259999999951</v>
+        <v>-35673.669999999984</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -1713,28 +1713,28 @@
         <v>10</v>
       </c>
       <c r="D14" s="9">
-        <v>334242.21000000002</v>
+        <v>334152.39</v>
       </c>
       <c r="E14" s="4"/>
       <c r="F14" s="10">
         <f>IF(C14&lt;=fact_months,"",ROUND(D14*(1+Equalisation!$G$8/100)+IF(C14&gt;=equalisation_month,Equalisation!$F$8,0),2))</f>
-        <v>337594.13</v>
+        <v>337503.42</v>
       </c>
       <c r="G14" s="10">
         <f t="shared" si="0"/>
-        <v>337594.13</v>
+        <v>337503.42</v>
       </c>
       <c r="H14" s="10">
         <f t="shared" si="1"/>
-        <v>3351.9199999999837</v>
+        <v>3351.0299999999697</v>
       </c>
       <c r="I14" s="14">
         <f t="shared" si="2"/>
-        <v>1.0028416219483421E-2</v>
+        <v>1.0028448397451144E-2</v>
       </c>
       <c r="J14" s="10">
         <f t="shared" si="3"/>
-        <v>-32331.339999999967</v>
+        <v>-32322.640000000014</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
@@ -1748,28 +1748,28 @@
         <v>11</v>
       </c>
       <c r="D15" s="9">
-        <v>336900.2</v>
+        <v>336809.67</v>
       </c>
       <c r="E15" s="4"/>
       <c r="F15" s="10">
         <f>IF(C15&lt;=fact_months,"",ROUND(D15*(1+Equalisation!$G$8/100)+IF(C15&gt;=equalisation_month,Equalisation!$F$8,0),2))</f>
-        <v>340213.82</v>
+        <v>340122.41</v>
       </c>
       <c r="G15" s="10">
         <f t="shared" si="0"/>
-        <v>340213.82</v>
+        <v>340122.41</v>
       </c>
       <c r="H15" s="10">
         <f t="shared" si="1"/>
-        <v>3313.6199999999953</v>
+        <v>3312.7399999999907</v>
       </c>
       <c r="I15" s="14">
         <f t="shared" si="2"/>
-        <v>9.8356130391136463E-3</v>
+        <v>9.83564397067338E-3</v>
       </c>
       <c r="J15" s="10">
         <f t="shared" si="3"/>
-        <v>-29017.719999999972</v>
+        <v>-29009.900000000023</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
@@ -1783,28 +1783,28 @@
         <v>12</v>
       </c>
       <c r="D16" s="9">
-        <v>337232.45</v>
+        <v>337141.83</v>
       </c>
       <c r="E16" s="4"/>
       <c r="F16" s="10">
         <f>IF(C16&lt;=fact_months,"",ROUND(D16*(1+Equalisation!$G$8/100)+IF(C16&gt;=equalisation_month,Equalisation!$F$8,0),2))</f>
-        <v>340541.29</v>
+        <v>340449.78</v>
       </c>
       <c r="G16" s="10">
         <f t="shared" si="0"/>
-        <v>340541.29</v>
+        <v>340449.78</v>
       </c>
       <c r="H16" s="10">
         <f t="shared" si="1"/>
-        <v>3308.8399999999674</v>
+        <v>3307.9500000000116</v>
       </c>
       <c r="I16" s="14">
         <f t="shared" si="2"/>
-        <v>9.8117485431783551E-3</v>
+        <v>9.8117459942600755E-3</v>
       </c>
       <c r="J16" s="10">
         <f t="shared" si="3"/>
-        <v>-25708.880000000005</v>
+        <v>-25701.950000000012</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
@@ -1818,10 +1818,10 @@
         <v>1</v>
       </c>
       <c r="D17" s="9">
-        <v>242838.79</v>
+        <v>242722.7</v>
       </c>
       <c r="E17" s="9">
-        <v>265129.15999999997</v>
+        <v>265002.40999999997</v>
       </c>
       <c r="F17" s="10" t="str">
         <f>IF(C17&lt;=fact_months,"",ROUND(D17*(1+Equalisation!$G$9/100)+IF(C17&gt;=equalisation_month,Equalisation!$F$9,0),2))</f>
@@ -1829,19 +1829,19 @@
       </c>
       <c r="G17" s="10">
         <f t="shared" si="0"/>
-        <v>265129.15999999997</v>
+        <v>265002.40999999997</v>
       </c>
       <c r="H17" s="10">
         <f t="shared" si="1"/>
-        <v>22290.369999999966</v>
+        <v>22279.709999999963</v>
       </c>
       <c r="I17" s="14">
         <f t="shared" si="2"/>
-        <v>9.1790813156332918E-2</v>
+        <v>9.179079665807921E-2</v>
       </c>
       <c r="J17" s="10">
         <f>H17</f>
-        <v>22290.369999999966</v>
+        <v>22279.709999999963</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
@@ -1855,10 +1855,10 @@
         <v>2</v>
       </c>
       <c r="D18" s="9">
-        <v>242136.94</v>
+        <v>242021.19</v>
       </c>
       <c r="E18" s="9">
-        <v>264282.53000000003</v>
+        <v>264156.19</v>
       </c>
       <c r="F18" s="10" t="str">
         <f>IF(C18&lt;=fact_months,"",ROUND(D18*(1+Equalisation!$G$9/100)+IF(C18&gt;=equalisation_month,Equalisation!$F$9,0),2))</f>
@@ -1866,19 +1866,19 @@
       </c>
       <c r="G18" s="10">
         <f t="shared" si="0"/>
-        <v>264282.53000000003</v>
+        <v>264156.19</v>
       </c>
       <c r="H18" s="10">
         <f t="shared" si="1"/>
-        <v>22145.590000000026</v>
+        <v>22135</v>
       </c>
       <c r="I18" s="14">
         <f t="shared" si="2"/>
-        <v>9.1458948808058882E-2</v>
+        <v>9.1458933823108629E-2</v>
       </c>
       <c r="J18" s="10">
         <f t="shared" ref="J18:J28" si="4">J17+H18</f>
-        <v>44435.959999999992</v>
+        <v>44414.709999999963</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
@@ -1892,10 +1892,10 @@
         <v>3</v>
       </c>
       <c r="D19" s="9">
-        <v>239095.61</v>
+        <v>238981.31</v>
       </c>
       <c r="E19" s="9">
-        <v>261059.03</v>
+        <v>260934.23</v>
       </c>
       <c r="F19" s="10" t="str">
         <f>IF(C19&lt;=fact_months,"",ROUND(D19*(1+Equalisation!$G$9/100)+IF(C19&gt;=equalisation_month,Equalisation!$F$9,0),2))</f>
@@ -1903,19 +1903,19 @@
       </c>
       <c r="G19" s="10">
         <f t="shared" si="0"/>
-        <v>261059.03</v>
+        <v>260934.23</v>
       </c>
       <c r="H19" s="10">
         <f t="shared" si="1"/>
-        <v>21963.420000000013</v>
+        <v>21952.920000000013</v>
       </c>
       <c r="I19" s="14">
         <f t="shared" si="2"/>
-        <v>9.1860406805461689E-2</v>
+        <v>9.1860405317888721E-2</v>
       </c>
       <c r="J19" s="10">
         <f t="shared" si="4"/>
-        <v>66399.38</v>
+        <v>66367.629999999976</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
@@ -1929,10 +1929,10 @@
         <v>4</v>
       </c>
       <c r="D20" s="9">
-        <v>235118.48</v>
+        <v>235006.07999999999</v>
       </c>
       <c r="E20" s="9">
-        <v>256678.84</v>
+        <v>256556.14</v>
       </c>
       <c r="F20" s="10" t="str">
         <f>IF(C20&lt;=fact_months,"",ROUND(D20*(1+Equalisation!$G$9/100)+IF(C20&gt;=equalisation_month,Equalisation!$F$9,0),2))</f>
@@ -1940,19 +1940,19 @@
       </c>
       <c r="G20" s="10">
         <f t="shared" si="0"/>
-        <v>256678.84</v>
+        <v>256556.14</v>
       </c>
       <c r="H20" s="10">
         <f t="shared" si="1"/>
-        <v>21560.359999999986</v>
+        <v>21550.060000000027</v>
       </c>
       <c r="I20" s="14">
         <f t="shared" si="2"/>
-        <v>9.1699980367344947E-2</v>
+        <v>9.170001048483524E-2</v>
       </c>
       <c r="J20" s="10">
         <f t="shared" si="4"/>
-        <v>87959.739999999991</v>
+        <v>87917.69</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
@@ -1966,10 +1966,10 @@
         <v>5</v>
       </c>
       <c r="D21" s="9">
-        <v>230673.45</v>
+        <v>230563.18</v>
       </c>
       <c r="E21" s="9">
-        <v>251975.28</v>
+        <v>251854.83</v>
       </c>
       <c r="F21" s="10" t="str">
         <f>IF(C21&lt;=fact_months,"",ROUND(D21*(1+Equalisation!$G$9/100)+IF(C21&gt;=equalisation_month,Equalisation!$F$9,0),2))</f>
@@ -1977,19 +1977,19 @@
       </c>
       <c r="G21" s="10">
         <f t="shared" si="0"/>
-        <v>251975.28</v>
+        <v>251854.83</v>
       </c>
       <c r="H21" s="10">
         <f t="shared" si="1"/>
-        <v>21301.829999999987</v>
+        <v>21291.649999999994</v>
       </c>
       <c r="I21" s="14">
         <f t="shared" si="2"/>
-        <v>9.2346258314513374E-2</v>
+        <v>9.2346271421134954E-2</v>
       </c>
       <c r="J21" s="10">
         <f t="shared" si="4"/>
-        <v>109261.56999999998</v>
+        <v>109209.34</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
@@ -2003,10 +2003,10 @@
         <v>6</v>
       </c>
       <c r="D22" s="9">
-        <v>226462.37</v>
+        <v>226354.11</v>
       </c>
       <c r="E22" s="9">
-        <v>247614.74</v>
+        <v>247496.37</v>
       </c>
       <c r="F22" s="10" t="str">
         <f>IF(C22&lt;=fact_months,"",ROUND(D22*(1+Equalisation!$G$9/100)+IF(C22&gt;=equalisation_month,Equalisation!$F$9,0),2))</f>
@@ -2014,19 +2014,19 @@
       </c>
       <c r="G22" s="10">
         <f t="shared" si="0"/>
-        <v>247614.74</v>
+        <v>247496.37</v>
       </c>
       <c r="H22" s="10">
         <f t="shared" si="1"/>
-        <v>21152.369999999995</v>
+        <v>21142.260000000009</v>
       </c>
       <c r="I22" s="14">
         <f t="shared" si="2"/>
-        <v>9.3403464778717971E-2</v>
+        <v>9.3403472991941738E-2</v>
       </c>
       <c r="J22" s="10">
         <f t="shared" si="4"/>
-        <v>130413.93999999997</v>
+        <v>130351.6</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
@@ -2040,10 +2040,10 @@
         <v>7</v>
       </c>
       <c r="D23" s="9">
-        <v>225058.68</v>
+        <v>224951.09</v>
       </c>
       <c r="E23" s="9">
-        <v>246001.24</v>
+        <v>245883.64</v>
       </c>
       <c r="F23" s="10" t="str">
         <f>IF(C23&lt;=fact_months,"",ROUND(D23*(1+Equalisation!$G$9/100)+IF(C23&gt;=equalisation_month,Equalisation!$F$9,0),2))</f>
@@ -2051,19 +2051,19 @@
       </c>
       <c r="G23" s="10">
         <f t="shared" si="0"/>
-        <v>246001.24</v>
+        <v>245883.64</v>
       </c>
       <c r="H23" s="10">
         <f t="shared" si="1"/>
-        <v>20942.559999999998</v>
+        <v>20932.550000000017</v>
       </c>
       <c r="I23" s="14">
         <f t="shared" si="2"/>
-        <v>9.3053776019658516E-2</v>
+        <v>9.3053783380200636E-2</v>
       </c>
       <c r="J23" s="10">
         <f t="shared" si="4"/>
-        <v>151356.49999999997</v>
+        <v>151284.15000000002</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
@@ -2077,10 +2077,10 @@
         <v>8</v>
       </c>
       <c r="D24" s="9">
-        <v>225526.58</v>
+        <v>225418.77</v>
       </c>
       <c r="E24" s="9">
-        <v>246679.43</v>
+        <v>246561.5</v>
       </c>
       <c r="F24" s="10" t="str">
         <f>IF(C24&lt;=fact_months,"",ROUND(D24*(1+Equalisation!$G$9/100)+IF(C24&gt;=equalisation_month,Equalisation!$F$9,0),2))</f>
@@ -2088,19 +2088,19 @@
       </c>
       <c r="G24" s="10">
         <f t="shared" si="0"/>
-        <v>246679.43</v>
+        <v>246561.5</v>
       </c>
       <c r="H24" s="10">
         <f t="shared" si="1"/>
-        <v>21152.850000000006</v>
+        <v>21142.73000000001</v>
       </c>
       <c r="I24" s="14">
         <f t="shared" si="2"/>
-        <v>9.3793157329836715E-2</v>
+        <v>9.3793121131838367E-2</v>
       </c>
       <c r="J24" s="10">
         <f t="shared" si="4"/>
-        <v>172509.34999999998</v>
+        <v>172426.88000000003</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
@@ -2114,28 +2114,28 @@
         <v>9</v>
       </c>
       <c r="D25" s="9">
-        <v>230439.5</v>
+        <v>230329.34</v>
       </c>
       <c r="E25" s="4"/>
       <c r="F25" s="10">
         <f>IF(C25&lt;=fact_months,"",ROUND(D25*(1+Equalisation!$G$9/100)+IF(C25&gt;=equalisation_month,Equalisation!$F$9,0),2))</f>
-        <v>262584.74</v>
+        <v>262446.38</v>
       </c>
       <c r="G25" s="10">
         <f t="shared" si="0"/>
-        <v>262584.74</v>
+        <v>262446.38</v>
       </c>
       <c r="H25" s="10">
         <f t="shared" si="1"/>
-        <v>32145.239999999991</v>
+        <v>32117.040000000008</v>
       </c>
       <c r="I25" s="14">
         <f t="shared" si="2"/>
-        <v>0.13949535561394635</v>
+        <v>0.13943963891009287</v>
       </c>
       <c r="J25" s="10">
         <f t="shared" si="4"/>
-        <v>204654.58999999997</v>
+        <v>204543.92000000004</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
@@ -2149,28 +2149,28 @@
         <v>10</v>
       </c>
       <c r="D26" s="9">
-        <v>235352.43</v>
+        <v>235239.92</v>
       </c>
       <c r="E26" s="4"/>
       <c r="F26" s="10">
         <f>IF(C26&lt;=fact_months,"",ROUND(D26*(1+Equalisation!$G$9/100)+IF(C26&gt;=equalisation_month,Equalisation!$F$9,0),2))</f>
-        <v>267952.28999999998</v>
+        <v>267811.37</v>
       </c>
       <c r="G26" s="10">
         <f t="shared" si="0"/>
-        <v>267952.28999999998</v>
+        <v>267811.37</v>
       </c>
       <c r="H26" s="10">
         <f t="shared" si="1"/>
-        <v>32599.859999999986</v>
+        <v>32571.449999999983</v>
       </c>
       <c r="I26" s="14">
         <f t="shared" si="2"/>
-        <v>0.13851507715471639</v>
+        <v>0.13846055550435479</v>
       </c>
       <c r="J26" s="10">
         <f t="shared" si="4"/>
-        <v>237254.44999999995</v>
+        <v>237115.37000000002</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
@@ -2184,28 +2184,28 @@
         <v>11</v>
       </c>
       <c r="D27" s="9">
-        <v>237224.02</v>
+        <v>237110.61</v>
       </c>
       <c r="E27" s="4"/>
       <c r="F27" s="10">
         <f>IF(C27&lt;=fact_months,"",ROUND(D27*(1+Equalisation!$G$9/100)+IF(C27&gt;=equalisation_month,Equalisation!$F$9,0),2))</f>
-        <v>269997.07</v>
+        <v>269855.15999999997</v>
       </c>
       <c r="G27" s="10">
         <f t="shared" si="0"/>
-        <v>269997.07</v>
+        <v>269855.15999999997</v>
       </c>
       <c r="H27" s="10">
         <f t="shared" si="1"/>
-        <v>32773.050000000017</v>
+        <v>32744.549999999988</v>
       </c>
       <c r="I27" s="14">
         <f t="shared" si="2"/>
-        <v>0.13815232538425079</v>
+        <v>0.13809820657118629</v>
       </c>
       <c r="J27" s="10">
         <f t="shared" si="4"/>
-        <v>270027.5</v>
+        <v>269859.92000000004</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
@@ -2219,28 +2219,28 @@
         <v>12</v>
       </c>
       <c r="D28" s="9">
-        <v>237457.97</v>
+        <v>237344.45</v>
       </c>
       <c r="E28" s="4"/>
       <c r="F28" s="10">
         <f>IF(C28&lt;=fact_months,"",ROUND(D28*(1+Equalisation!$G$9/100)+IF(C28&gt;=equalisation_month,Equalisation!$F$9,0),2))</f>
-        <v>270252.65999999997</v>
+        <v>270110.64</v>
       </c>
       <c r="G28" s="10">
         <f t="shared" si="0"/>
-        <v>270252.65999999997</v>
+        <v>270110.64</v>
       </c>
       <c r="H28" s="10">
         <f t="shared" si="1"/>
-        <v>32794.689999999973</v>
+        <v>32766.190000000002</v>
       </c>
       <c r="I28" s="14">
         <f t="shared" si="2"/>
-        <v>0.13810734590209783</v>
+        <v>0.13805332292370856</v>
       </c>
       <c r="J28" s="10">
         <f t="shared" si="4"/>
-        <v>302822.18999999994</v>
+        <v>302626.11000000004</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
@@ -2254,10 +2254,10 @@
         <v>1</v>
       </c>
       <c r="D29" s="9">
-        <v>228283.47</v>
+        <v>228268.11</v>
       </c>
       <c r="E29" s="9">
-        <v>231390.85</v>
+        <v>231375.28</v>
       </c>
       <c r="F29" s="10" t="str">
         <f>IF(C29&lt;=fact_months,"",ROUND(D29*(1+Equalisation!$G$10/100)+IF(C29&gt;=equalisation_month,Equalisation!$F$10,0),2))</f>
@@ -2265,19 +2265,19 @@
       </c>
       <c r="G29" s="10">
         <f t="shared" si="0"/>
-        <v>231390.85</v>
+        <v>231375.28</v>
       </c>
       <c r="H29" s="10">
         <f t="shared" si="1"/>
-        <v>3107.3800000000047</v>
+        <v>3107.1700000000128</v>
       </c>
       <c r="I29" s="14">
         <f t="shared" si="2"/>
-        <v>1.361193607228769E-2</v>
+        <v>1.3611932039039588E-2</v>
       </c>
       <c r="J29" s="10">
         <f>H29</f>
-        <v>3107.3800000000047</v>
+        <v>3107.1700000000128</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
@@ -2291,10 +2291,10 @@
         <v>2</v>
       </c>
       <c r="D30" s="9">
-        <v>227623.69</v>
+        <v>227608.38</v>
       </c>
       <c r="E30" s="9">
-        <v>230690.86</v>
+        <v>230675.34</v>
       </c>
       <c r="F30" s="10" t="str">
         <f>IF(C30&lt;=fact_months,"",ROUND(D30*(1+Equalisation!$G$10/100)+IF(C30&gt;=equalisation_month,Equalisation!$F$10,0),2))</f>
@@ -2302,19 +2302,19 @@
       </c>
       <c r="G30" s="10">
         <f t="shared" si="0"/>
-        <v>230690.86</v>
+        <v>230675.34</v>
       </c>
       <c r="H30" s="10">
         <f t="shared" si="1"/>
-        <v>3067.1699999999837</v>
+        <v>3066.9599999999919</v>
       </c>
       <c r="I30" s="14">
         <f t="shared" si="2"/>
-        <v>1.3474739821676662E-2</v>
+        <v>1.347472355806931E-2</v>
       </c>
       <c r="J30" s="10">
         <f t="shared" ref="J30:J40" si="5">J29+H30</f>
-        <v>6174.5499999999884</v>
+        <v>6174.1300000000047</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
@@ -2328,10 +2328,10 @@
         <v>3</v>
       </c>
       <c r="D31" s="9">
-        <v>224764.65</v>
+        <v>224749.53</v>
       </c>
       <c r="E31" s="9">
-        <v>227525.39</v>
+        <v>227510.09</v>
       </c>
       <c r="F31" s="10" t="str">
         <f>IF(C31&lt;=fact_months,"",ROUND(D31*(1+Equalisation!$G$10/100)+IF(C31&gt;=equalisation_month,Equalisation!$F$10,0),2))</f>
@@ -2339,19 +2339,19 @@
       </c>
       <c r="G31" s="10">
         <f t="shared" si="0"/>
-        <v>227525.39</v>
+        <v>227510.09</v>
       </c>
       <c r="H31" s="10">
         <f t="shared" si="1"/>
-        <v>2760.7400000000198</v>
+        <v>2760.5599999999977</v>
       </c>
       <c r="I31" s="14">
         <f t="shared" si="2"/>
-        <v>1.2282803367878445E-2</v>
+        <v>1.2282828800576347E-2</v>
       </c>
       <c r="J31" s="10">
         <f t="shared" si="5"/>
-        <v>8935.2900000000081</v>
+        <v>8934.6900000000023</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
@@ -2365,10 +2365,10 @@
         <v>4</v>
       </c>
       <c r="D32" s="9">
-        <v>221025.9</v>
+        <v>221011.03</v>
       </c>
       <c r="E32" s="9">
-        <v>224049.75</v>
+        <v>224034.68</v>
       </c>
       <c r="F32" s="10" t="str">
         <f>IF(C32&lt;=fact_months,"",ROUND(D32*(1+Equalisation!$G$10/100)+IF(C32&gt;=equalisation_month,Equalisation!$F$10,0),2))</f>
@@ -2376,19 +2376,19 @@
       </c>
       <c r="G32" s="10">
         <f t="shared" si="0"/>
-        <v>224049.75</v>
+        <v>224034.68</v>
       </c>
       <c r="H32" s="10">
         <f t="shared" si="1"/>
-        <v>3023.8500000000058</v>
+        <v>3023.6499999999942</v>
       </c>
       <c r="I32" s="14">
         <f t="shared" si="2"/>
-        <v>1.3680975849436677E-2</v>
+        <v>1.3680991396673706E-2</v>
       </c>
       <c r="J32" s="10">
         <f t="shared" si="5"/>
-        <v>11959.140000000014</v>
+        <v>11958.339999999997</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
@@ -2402,10 +2402,10 @@
         <v>5</v>
       </c>
       <c r="D33" s="9">
-        <v>216847.3</v>
+        <v>216832.72</v>
       </c>
       <c r="E33" s="9">
-        <v>219787.72</v>
+        <v>219772.95</v>
       </c>
       <c r="F33" s="10" t="str">
         <f>IF(C33&lt;=fact_months,"",ROUND(D33*(1+Equalisation!$G$10/100)+IF(C33&gt;=equalisation_month,Equalisation!$F$10,0),2))</f>
@@ -2413,19 +2413,19 @@
       </c>
       <c r="G33" s="10">
         <f t="shared" si="0"/>
-        <v>219787.72</v>
+        <v>219772.95</v>
       </c>
       <c r="H33" s="10">
         <f t="shared" si="1"/>
-        <v>2940.4200000000128</v>
+        <v>2940.2300000000105</v>
       </c>
       <c r="I33" s="14">
         <f t="shared" si="2"/>
-        <v>1.3559864476062247E-2</v>
+        <v>1.3559900000332102E-2</v>
       </c>
       <c r="J33" s="10">
         <f t="shared" si="5"/>
-        <v>14899.560000000027</v>
+        <v>14898.570000000007</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
@@ -2439,10 +2439,10 @@
         <v>6</v>
       </c>
       <c r="D34" s="9">
-        <v>212888.63</v>
+        <v>212874.31</v>
       </c>
       <c r="E34" s="9">
-        <v>216019.66</v>
+        <v>216005.13</v>
       </c>
       <c r="F34" s="10" t="str">
         <f>IF(C34&lt;=fact_months,"",ROUND(D34*(1+Equalisation!$G$10/100)+IF(C34&gt;=equalisation_month,Equalisation!$F$10,0),2))</f>
@@ -2450,19 +2450,19 @@
       </c>
       <c r="G34" s="10">
         <f t="shared" si="0"/>
-        <v>216019.66</v>
+        <v>216005.13</v>
       </c>
       <c r="H34" s="10">
         <f t="shared" si="1"/>
-        <v>3131.0299999999988</v>
+        <v>3130.820000000007</v>
       </c>
       <c r="I34" s="14">
         <f t="shared" si="2"/>
-        <v>1.4707361309056283E-2</v>
+        <v>1.4707364171843972E-2</v>
       </c>
       <c r="J34" s="10">
         <f t="shared" si="5"/>
-        <v>18030.590000000026</v>
+        <v>18029.390000000014</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
@@ -2476,10 +2476,10 @@
         <v>7</v>
       </c>
       <c r="D35" s="9">
-        <v>211569.07</v>
+        <v>211554.84</v>
       </c>
       <c r="E35" s="9">
-        <v>214065.27</v>
+        <v>214050.87</v>
       </c>
       <c r="F35" s="10" t="str">
         <f>IF(C35&lt;=fact_months,"",ROUND(D35*(1+Equalisation!$G$10/100)+IF(C35&gt;=equalisation_month,Equalisation!$F$10,0),2))</f>
@@ -2487,19 +2487,19 @@
       </c>
       <c r="G35" s="10">
         <f t="shared" si="0"/>
-        <v>214065.27</v>
+        <v>214050.87</v>
       </c>
       <c r="H35" s="10">
         <f t="shared" si="1"/>
-        <v>2496.1999999999825</v>
+        <v>2496.0299999999988</v>
       </c>
       <c r="I35" s="14">
         <f t="shared" si="2"/>
-        <v>1.1798511001631677E-2</v>
+        <v>1.1798501041148475E-2</v>
       </c>
       <c r="J35" s="10">
         <f t="shared" si="5"/>
-        <v>20526.790000000008</v>
+        <v>20525.420000000013</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
@@ -2513,10 +2513,10 @@
         <v>8</v>
       </c>
       <c r="D36" s="9">
-        <v>212008.92</v>
+        <v>211994.66</v>
       </c>
       <c r="E36" s="9">
-        <v>214745.39</v>
+        <v>214730.95</v>
       </c>
       <c r="F36" s="10" t="str">
         <f>IF(C36&lt;=fact_months,"",ROUND(D36*(1+Equalisation!$G$10/100)+IF(C36&gt;=equalisation_month,Equalisation!$F$10,0),2))</f>
@@ -2524,19 +2524,19 @@
       </c>
       <c r="G36" s="10">
         <f t="shared" si="0"/>
-        <v>214745.39</v>
+        <v>214730.95</v>
       </c>
       <c r="H36" s="10">
         <f t="shared" si="1"/>
-        <v>2736.4700000000012</v>
+        <v>2736.2900000000081</v>
       </c>
       <c r="I36" s="14">
         <f t="shared" si="2"/>
-        <v>1.290733427631253E-2</v>
+        <v>1.2907353421072059E-2</v>
       </c>
       <c r="J36" s="10">
         <f t="shared" si="5"/>
-        <v>23263.260000000009</v>
+        <v>23261.710000000021</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
@@ -2550,28 +2550,28 @@
         <v>9</v>
       </c>
       <c r="D37" s="9">
-        <v>216627.38</v>
+        <v>216612.8</v>
       </c>
       <c r="E37" s="4"/>
       <c r="F37" s="10">
         <f>IF(C37&lt;=fact_months,"",ROUND(D37*(1+Equalisation!$G$10/100)+IF(C37&gt;=equalisation_month,Equalisation!$F$10,0),2))</f>
-        <v>221281.25</v>
+        <v>221266.48</v>
       </c>
       <c r="G37" s="10">
         <f t="shared" ref="G37:G68" si="6">IF(C37&lt;=fact_months,E37,F37)</f>
-        <v>221281.25</v>
+        <v>221266.48</v>
       </c>
       <c r="H37" s="10">
         <f t="shared" ref="H37:H68" si="7">G37-D37</f>
-        <v>4653.8699999999953</v>
+        <v>4653.6800000000221</v>
       </c>
       <c r="I37" s="14">
         <f t="shared" ref="I37:I68" si="8">IF(D37=0,"",H37/D37)</f>
-        <v>2.1483295417227478E-2</v>
+        <v>2.1483864296108181E-2</v>
       </c>
       <c r="J37" s="10">
         <f t="shared" si="5"/>
-        <v>27917.130000000005</v>
+        <v>27915.390000000043</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
@@ -2585,28 +2585,28 @@
         <v>10</v>
       </c>
       <c r="D38" s="9">
-        <v>221245.83</v>
+        <v>221230.95</v>
       </c>
       <c r="E38" s="4"/>
       <c r="F38" s="10">
         <f>IF(C38&lt;=fact_months,"",ROUND(D38*(1+Equalisation!$G$10/100)+IF(C38&gt;=equalisation_month,Equalisation!$F$10,0),2))</f>
-        <v>225961.01</v>
+        <v>225945.93</v>
       </c>
       <c r="G38" s="10">
         <f t="shared" si="6"/>
-        <v>225961.01</v>
+        <v>225945.93</v>
       </c>
       <c r="H38" s="10">
         <f t="shared" si="7"/>
-        <v>4715.1800000000221</v>
+        <v>4714.9799999999814</v>
       </c>
       <c r="I38" s="14">
         <f t="shared" si="8"/>
-        <v>2.1311949698667867E-2</v>
+        <v>2.1312479108370603E-2</v>
       </c>
       <c r="J38" s="10">
         <f t="shared" si="5"/>
-        <v>32632.310000000027</v>
+        <v>32630.370000000024</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
@@ -2620,28 +2620,28 @@
         <v>11</v>
       </c>
       <c r="D39" s="9">
-        <v>223005.24</v>
+        <v>222990.24</v>
       </c>
       <c r="E39" s="4"/>
       <c r="F39" s="10">
         <f>IF(C39&lt;=fact_months,"",ROUND(D39*(1+Equalisation!$G$10/100)+IF(C39&gt;=equalisation_month,Equalisation!$F$10,0),2))</f>
-        <v>227743.78</v>
+        <v>227728.58</v>
       </c>
       <c r="G39" s="10">
         <f t="shared" si="6"/>
-        <v>227743.78</v>
+        <v>227728.58</v>
       </c>
       <c r="H39" s="10">
         <f t="shared" si="7"/>
-        <v>4738.5400000000081</v>
+        <v>4738.3399999999965</v>
       </c>
       <c r="I39" s="14">
         <f t="shared" si="8"/>
-        <v>2.1248559002470115E-2</v>
+        <v>2.1249091440055837E-2</v>
       </c>
       <c r="J39" s="10">
         <f t="shared" si="5"/>
-        <v>37370.850000000035</v>
+        <v>37368.710000000021</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
@@ -2655,28 +2655,28 @@
         <v>12</v>
       </c>
       <c r="D40" s="9">
-        <v>223225.16</v>
+        <v>223210.15</v>
       </c>
       <c r="E40" s="4"/>
       <c r="F40" s="10">
         <f>IF(C40&lt;=fact_months,"",ROUND(D40*(1+Equalisation!$G$10/100)+IF(C40&gt;=equalisation_month,Equalisation!$F$10,0),2))</f>
-        <v>227966.61</v>
+        <v>227951.41</v>
       </c>
       <c r="G40" s="10">
         <f t="shared" si="6"/>
-        <v>227966.61</v>
+        <v>227951.41</v>
       </c>
       <c r="H40" s="10">
         <f t="shared" si="7"/>
-        <v>4741.4499999999825</v>
+        <v>4741.2600000000093</v>
       </c>
       <c r="I40" s="14">
         <f t="shared" si="8"/>
-        <v>2.1240661222955256E-2</v>
+        <v>2.1241238357664335E-2</v>
       </c>
       <c r="J40" s="10">
         <f t="shared" si="5"/>
-        <v>42112.300000000017</v>
+        <v>42109.97000000003</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
@@ -2690,10 +2690,10 @@
         <v>1</v>
       </c>
       <c r="D41" s="9">
-        <v>218086.63</v>
+        <v>218080.32</v>
       </c>
       <c r="E41" s="9">
-        <v>223337.15</v>
+        <v>223330.68</v>
       </c>
       <c r="F41" s="10" t="str">
         <f>IF(C41&lt;=fact_months,"",ROUND(D41*(1+Equalisation!$G$11/100)+IF(C41&gt;=equalisation_month,Equalisation!$F$11,0),2))</f>
@@ -2701,19 +2701,19 @@
       </c>
       <c r="G41" s="10">
         <f t="shared" si="6"/>
-        <v>223337.15</v>
+        <v>223330.68</v>
       </c>
       <c r="H41" s="10">
         <f t="shared" si="7"/>
-        <v>5250.5199999999895</v>
+        <v>5250.359999999986</v>
       </c>
       <c r="I41" s="14">
         <f t="shared" si="8"/>
-        <v>2.4075386923077261E-2</v>
+        <v>2.4075349852751435E-2</v>
       </c>
       <c r="J41" s="10">
         <f>H41</f>
-        <v>5250.5199999999895</v>
+        <v>5250.359999999986</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
@@ -2727,10 +2727,10 @@
         <v>2</v>
       </c>
       <c r="D42" s="9">
-        <v>217456.32</v>
+        <v>217450.03</v>
       </c>
       <c r="E42" s="9">
-        <v>222421.91</v>
+        <v>222415.48</v>
       </c>
       <c r="F42" s="10" t="str">
         <f>IF(C42&lt;=fact_months,"",ROUND(D42*(1+Equalisation!$G$11/100)+IF(C42&gt;=equalisation_month,Equalisation!$F$11,0),2))</f>
@@ -2738,19 +2738,19 @@
       </c>
       <c r="G42" s="10">
         <f t="shared" si="6"/>
-        <v>222421.91</v>
+        <v>222415.48</v>
       </c>
       <c r="H42" s="10">
         <f t="shared" si="7"/>
-        <v>4965.5899999999965</v>
+        <v>4965.4500000000116</v>
       </c>
       <c r="I42" s="14">
         <f t="shared" si="8"/>
-        <v>2.28348847253554E-2</v>
+        <v>2.2834901425398801E-2</v>
       </c>
       <c r="J42" s="10">
         <f t="shared" ref="J42:J52" si="9">J41+H42</f>
-        <v>10216.109999999986</v>
+        <v>10215.809999999998</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
@@ -2764,10 +2764,10 @@
         <v>3</v>
       </c>
       <c r="D43" s="9">
-        <v>214724.99</v>
+        <v>214718.77</v>
       </c>
       <c r="E43" s="9">
-        <v>220098.35</v>
+        <v>220091.97</v>
       </c>
       <c r="F43" s="10" t="str">
         <f>IF(C43&lt;=fact_months,"",ROUND(D43*(1+Equalisation!$G$11/100)+IF(C43&gt;=equalisation_month,Equalisation!$F$11,0),2))</f>
@@ -2775,19 +2775,19 @@
       </c>
       <c r="G43" s="10">
         <f t="shared" si="6"/>
-        <v>220098.35</v>
+        <v>220091.97</v>
       </c>
       <c r="H43" s="10">
         <f t="shared" si="7"/>
-        <v>5373.3600000000151</v>
+        <v>5373.2000000000116</v>
       </c>
       <c r="I43" s="14">
         <f t="shared" si="8"/>
-        <v>2.5024381186372464E-2</v>
+        <v>2.5024360935003549E-2</v>
       </c>
       <c r="J43" s="10">
         <f t="shared" si="9"/>
-        <v>15589.470000000001</v>
+        <v>15589.010000000009</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
@@ -2801,10 +2801,10 @@
         <v>4</v>
       </c>
       <c r="D44" s="9">
-        <v>211153.24</v>
+        <v>211147.13</v>
       </c>
       <c r="E44" s="9">
-        <v>215948.78</v>
+        <v>215942.53</v>
       </c>
       <c r="F44" s="10" t="str">
         <f>IF(C44&lt;=fact_months,"",ROUND(D44*(1+Equalisation!$G$11/100)+IF(C44&gt;=equalisation_month,Equalisation!$F$11,0),2))</f>
@@ -2812,19 +2812,19 @@
       </c>
       <c r="G44" s="10">
         <f t="shared" si="6"/>
-        <v>215948.78</v>
+        <v>215942.53</v>
       </c>
       <c r="H44" s="10">
         <f t="shared" si="7"/>
-        <v>4795.5400000000081</v>
+        <v>4795.3999999999942</v>
       </c>
       <c r="I44" s="14">
         <f t="shared" si="8"/>
-        <v>2.2711183593488827E-2</v>
+        <v>2.2711177746057899E-2</v>
       </c>
       <c r="J44" s="10">
         <f t="shared" si="9"/>
-        <v>20385.010000000009</v>
+        <v>20384.410000000003</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
@@ -2838,10 +2838,10 @@
         <v>5</v>
       </c>
       <c r="D45" s="9">
-        <v>207161.29</v>
+        <v>207155.29</v>
       </c>
       <c r="E45" s="9">
-        <v>212017.25</v>
+        <v>212011.11</v>
       </c>
       <c r="F45" s="10" t="str">
         <f>IF(C45&lt;=fact_months,"",ROUND(D45*(1+Equalisation!$G$11/100)+IF(C45&gt;=equalisation_month,Equalisation!$F$11,0),2))</f>
@@ -2849,19 +2849,19 @@
       </c>
       <c r="G45" s="10">
         <f t="shared" si="6"/>
-        <v>212017.25</v>
+        <v>212011.11</v>
       </c>
       <c r="H45" s="10">
         <f t="shared" si="7"/>
-        <v>4855.9599999999919</v>
+        <v>4855.8199999999779</v>
       </c>
       <c r="I45" s="14">
         <f t="shared" si="8"/>
-        <v>2.3440479637870527E-2</v>
+        <v>2.3440482741232328E-2</v>
       </c>
       <c r="J45" s="10">
         <f t="shared" si="9"/>
-        <v>25240.97</v>
+        <v>25240.229999999981</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
@@ -2875,10 +2875,10 @@
         <v>6</v>
       </c>
       <c r="D46" s="9">
-        <v>203379.44</v>
+        <v>203373.55</v>
       </c>
       <c r="E46" s="9">
-        <v>208172.39</v>
+        <v>208166.37</v>
       </c>
       <c r="F46" s="10" t="str">
         <f>IF(C46&lt;=fact_months,"",ROUND(D46*(1+Equalisation!$G$11/100)+IF(C46&gt;=equalisation_month,Equalisation!$F$11,0),2))</f>
@@ -2886,19 +2886,19 @@
       </c>
       <c r="G46" s="10">
         <f t="shared" si="6"/>
-        <v>208172.39</v>
+        <v>208166.37</v>
       </c>
       <c r="H46" s="10">
         <f t="shared" si="7"/>
-        <v>4792.9500000000116</v>
+        <v>4792.820000000007</v>
       </c>
       <c r="I46" s="14">
         <f t="shared" si="8"/>
-        <v>2.3566541436046886E-2</v>
+        <v>2.3566584740247722E-2</v>
       </c>
       <c r="J46" s="10">
         <f t="shared" si="9"/>
-        <v>30033.920000000013</v>
+        <v>30033.049999999988</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
@@ -2912,10 +2912,10 @@
         <v>7</v>
       </c>
       <c r="D47" s="9">
-        <v>202118.83</v>
+        <v>202112.97</v>
       </c>
       <c r="E47" s="9">
-        <v>206780.17</v>
+        <v>206774.17</v>
       </c>
       <c r="F47" s="10" t="str">
         <f>IF(C47&lt;=fact_months,"",ROUND(D47*(1+Equalisation!$G$11/100)+IF(C47&gt;=equalisation_month,Equalisation!$F$11,0),2))</f>
@@ -2923,19 +2923,19 @@
       </c>
       <c r="G47" s="10">
         <f t="shared" si="6"/>
-        <v>206780.17</v>
+        <v>206774.17</v>
       </c>
       <c r="H47" s="10">
         <f t="shared" si="7"/>
-        <v>4661.3400000000256</v>
+        <v>4661.2000000000116</v>
       </c>
       <c r="I47" s="14">
         <f t="shared" si="8"/>
-        <v>2.3062373753103688E-2</v>
+        <v>2.3062349734408492E-2</v>
       </c>
       <c r="J47" s="10">
         <f t="shared" si="9"/>
-        <v>34695.260000000038</v>
+        <v>34694.25</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
@@ -2949,10 +2949,10 @@
         <v>8</v>
       </c>
       <c r="D48" s="9">
-        <v>202539.03</v>
+        <v>202533.16</v>
       </c>
       <c r="E48" s="9">
-        <v>207579.41</v>
+        <v>207573.4</v>
       </c>
       <c r="F48" s="10" t="str">
         <f>IF(C48&lt;=fact_months,"",ROUND(D48*(1+Equalisation!$G$11/100)+IF(C48&gt;=equalisation_month,Equalisation!$F$11,0),2))</f>
@@ -2960,19 +2960,19 @@
       </c>
       <c r="G48" s="10">
         <f t="shared" si="6"/>
-        <v>207579.41</v>
+        <v>207573.4</v>
       </c>
       <c r="H48" s="10">
         <f t="shared" si="7"/>
-        <v>5040.3800000000047</v>
+        <v>5040.2399999999907</v>
       </c>
       <c r="I48" s="14">
         <f t="shared" si="8"/>
-        <v>2.488596889202049E-2</v>
+        <v>2.4885998914943069E-2</v>
       </c>
       <c r="J48" s="10">
         <f t="shared" si="9"/>
-        <v>39735.640000000043</v>
+        <v>39734.489999999991</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
@@ -2986,28 +2986,28 @@
         <v>9</v>
       </c>
       <c r="D49" s="9">
-        <v>206951.19</v>
+        <v>206945.19</v>
       </c>
       <c r="E49" s="4"/>
       <c r="F49" s="10">
         <f>IF(C49&lt;=fact_months,"",ROUND(D49*(1+Equalisation!$G$11/100)+IF(C49&gt;=equalisation_month,Equalisation!$F$11,0),2))</f>
-        <v>219056.5</v>
+        <v>219050.36</v>
       </c>
       <c r="G49" s="10">
         <f t="shared" si="6"/>
-        <v>219056.5</v>
+        <v>219050.36</v>
       </c>
       <c r="H49" s="10">
         <f t="shared" si="7"/>
-        <v>12105.309999999998</v>
+        <v>12105.169999999984</v>
       </c>
       <c r="I49" s="14">
         <f t="shared" si="8"/>
-        <v>5.8493551063900612E-2</v>
+        <v>5.8494570470567511E-2</v>
       </c>
       <c r="J49" s="10">
         <f t="shared" si="9"/>
-        <v>51840.950000000041</v>
+        <v>51839.659999999974</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
@@ -3021,28 +3021,28 @@
         <v>10</v>
       </c>
       <c r="D50" s="9">
-        <v>211363.35</v>
+        <v>211357.22</v>
       </c>
       <c r="E50" s="4"/>
       <c r="F50" s="10">
         <f>IF(C50&lt;=fact_months,"",ROUND(D50*(1+Equalisation!$G$11/100)+IF(C50&gt;=equalisation_month,Equalisation!$F$11,0),2))</f>
-        <v>223572.6</v>
+        <v>223566.33</v>
       </c>
       <c r="G50" s="10">
         <f t="shared" si="6"/>
-        <v>223572.6</v>
+        <v>223566.33</v>
       </c>
       <c r="H50" s="10">
         <f t="shared" si="7"/>
-        <v>12209.25</v>
+        <v>12209.109999999986</v>
       </c>
       <c r="I50" s="14">
         <f t="shared" si="8"/>
-        <v>5.7764271809658582E-2</v>
+        <v>5.776528476292405E-2</v>
       </c>
       <c r="J50" s="10">
         <f t="shared" si="9"/>
-        <v>64050.200000000041</v>
+        <v>64048.76999999996</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
@@ -3056,28 +3056,28 @@
         <v>11</v>
       </c>
       <c r="D51" s="9">
-        <v>213044.17</v>
+        <v>213038</v>
       </c>
       <c r="E51" s="4"/>
       <c r="F51" s="10">
         <f>IF(C51&lt;=fact_months,"",ROUND(D51*(1+Equalisation!$G$11/100)+IF(C51&gt;=equalisation_month,Equalisation!$F$11,0),2))</f>
-        <v>225293.02</v>
+        <v>225286.7</v>
       </c>
       <c r="G51" s="10">
         <f t="shared" si="6"/>
-        <v>225293.02</v>
+        <v>225286.7</v>
       </c>
       <c r="H51" s="10">
         <f t="shared" si="7"/>
-        <v>12248.849999999977</v>
+        <v>12248.700000000012</v>
       </c>
       <c r="I51" s="14">
         <f t="shared" si="8"/>
-        <v>5.7494415359969603E-2</v>
+        <v>5.7495376411720027E-2</v>
       </c>
       <c r="J51" s="10">
         <f t="shared" si="9"/>
-        <v>76299.050000000017</v>
+        <v>76297.469999999972</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
@@ -3091,28 +3091,28 @@
         <v>12</v>
       </c>
       <c r="D52" s="9">
-        <v>213254.27</v>
+        <v>213248.09</v>
       </c>
       <c r="E52" s="4"/>
       <c r="F52" s="10">
         <f>IF(C52&lt;=fact_months,"",ROUND(D52*(1+Equalisation!$G$11/100)+IF(C52&gt;=equalisation_month,Equalisation!$F$11,0),2))</f>
-        <v>225508.07</v>
+        <v>225501.74</v>
       </c>
       <c r="G52" s="10">
         <f t="shared" si="6"/>
-        <v>225508.07</v>
+        <v>225501.74</v>
       </c>
       <c r="H52" s="10">
         <f t="shared" si="7"/>
-        <v>12253.800000000017</v>
+        <v>12253.649999999994</v>
       </c>
       <c r="I52" s="14">
         <f t="shared" si="8"/>
-        <v>5.746098307902589E-2</v>
+        <v>5.7461944911206445E-2</v>
       </c>
       <c r="J52" s="10">
         <f t="shared" si="9"/>
-        <v>88552.850000000035</v>
+        <v>88551.119999999966</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
@@ -3126,10 +3126,10 @@
         <v>1</v>
       </c>
       <c r="D53" s="9">
-        <v>201200.07</v>
+        <v>201149.39</v>
       </c>
       <c r="E53" s="9">
-        <v>206080.7</v>
+        <v>206028.79</v>
       </c>
       <c r="F53" s="10" t="str">
         <f>IF(C53&lt;=fact_months,"",ROUND(D53*(1+Equalisation!$G$12/100)+IF(C53&gt;=equalisation_month,Equalisation!$F$12,0),2))</f>
@@ -3137,19 +3137,19 @@
       </c>
       <c r="G53" s="10">
         <f t="shared" si="6"/>
-        <v>206080.7</v>
+        <v>206028.79</v>
       </c>
       <c r="H53" s="10">
         <f t="shared" si="7"/>
-        <v>4880.6300000000047</v>
+        <v>4879.3999999999942</v>
       </c>
       <c r="I53" s="14">
         <f t="shared" si="8"/>
-        <v>2.4257595934236029E-2</v>
+        <v>2.4257592826903398E-2</v>
       </c>
       <c r="J53" s="10">
         <f>H53</f>
-        <v>4880.6300000000047</v>
+        <v>4879.3999999999942</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.3">
@@ -3163,10 +3163,10 @@
         <v>2</v>
       </c>
       <c r="D54" s="9">
-        <v>200618.57</v>
+        <v>200568.03</v>
       </c>
       <c r="E54" s="9">
-        <v>205606.17</v>
+        <v>205554.38</v>
       </c>
       <c r="F54" s="10" t="str">
         <f>IF(C54&lt;=fact_months,"",ROUND(D54*(1+Equalisation!$G$12/100)+IF(C54&gt;=equalisation_month,Equalisation!$F$12,0),2))</f>
@@ -3174,19 +3174,19 @@
       </c>
       <c r="G54" s="10">
         <f t="shared" si="6"/>
-        <v>205606.17</v>
+        <v>205554.38</v>
       </c>
       <c r="H54" s="10">
         <f t="shared" si="7"/>
-        <v>4987.6000000000058</v>
+        <v>4986.3500000000058</v>
       </c>
       <c r="I54" s="14">
         <f t="shared" si="8"/>
-        <v>2.4861108321129026E-2</v>
+        <v>2.4861140631435658E-2</v>
       </c>
       <c r="J54" s="10">
         <f t="shared" ref="J54:J64" si="10">J53+H54</f>
-        <v>9868.2300000000105</v>
+        <v>9865.75</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
@@ -3200,10 +3200,10 @@
         <v>3</v>
       </c>
       <c r="D55" s="9">
-        <v>198098.72</v>
+        <v>198048.82</v>
       </c>
       <c r="E55" s="9">
-        <v>202981.89</v>
+        <v>202930.76</v>
       </c>
       <c r="F55" s="10" t="str">
         <f>IF(C55&lt;=fact_months,"",ROUND(D55*(1+Equalisation!$G$12/100)+IF(C55&gt;=equalisation_month,Equalisation!$F$12,0),2))</f>
@@ -3211,19 +3211,19 @@
       </c>
       <c r="G55" s="10">
         <f t="shared" si="6"/>
-        <v>202981.89</v>
+        <v>202930.76</v>
       </c>
       <c r="H55" s="10">
         <f t="shared" si="7"/>
-        <v>4883.1700000000128</v>
+        <v>4881.9400000000023</v>
       </c>
       <c r="I55" s="14">
         <f t="shared" si="8"/>
-        <v>2.4650184514064567E-2</v>
+        <v>2.4650184737278424E-2</v>
       </c>
       <c r="J55" s="10">
         <f t="shared" si="10"/>
-        <v>14751.400000000023</v>
+        <v>14747.690000000002</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
@@ -3237,10 +3237,10 @@
         <v>4</v>
       </c>
       <c r="D56" s="9">
-        <v>194803.54</v>
+        <v>194754.46</v>
       </c>
       <c r="E56" s="9">
-        <v>199767.23</v>
+        <v>199716.9</v>
       </c>
       <c r="F56" s="10" t="str">
         <f>IF(C56&lt;=fact_months,"",ROUND(D56*(1+Equalisation!$G$12/100)+IF(C56&gt;=equalisation_month,Equalisation!$F$12,0),2))</f>
@@ -3248,19 +3248,19 @@
       </c>
       <c r="G56" s="10">
         <f t="shared" si="6"/>
-        <v>199767.23</v>
+        <v>199716.9</v>
       </c>
       <c r="H56" s="10">
         <f t="shared" si="7"/>
-        <v>4963.6900000000023</v>
+        <v>4962.4400000000023</v>
       </c>
       <c r="I56" s="14">
         <f t="shared" si="8"/>
-        <v>2.5480491781617532E-2</v>
+        <v>2.5480494772751303E-2</v>
       </c>
       <c r="J56" s="10">
         <f t="shared" si="10"/>
-        <v>19715.090000000026</v>
+        <v>19710.130000000005</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
@@ -3274,10 +3274,10 @@
         <v>5</v>
       </c>
       <c r="D57" s="9">
-        <v>191120.69</v>
+        <v>191072.54</v>
       </c>
       <c r="E57" s="9">
-        <v>195988.38</v>
+        <v>195939</v>
       </c>
       <c r="F57" s="10" t="str">
         <f>IF(C57&lt;=fact_months,"",ROUND(D57*(1+Equalisation!$G$12/100)+IF(C57&gt;=equalisation_month,Equalisation!$F$12,0),2))</f>
@@ -3285,19 +3285,19 @@
       </c>
       <c r="G57" s="10">
         <f t="shared" si="6"/>
-        <v>195988.38</v>
+        <v>195939</v>
       </c>
       <c r="H57" s="10">
         <f t="shared" si="7"/>
-        <v>4867.6900000000023</v>
+        <v>4866.4599999999919</v>
       </c>
       <c r="I57" s="14">
         <f t="shared" si="8"/>
-        <v>2.5469194360903585E-2</v>
+        <v>2.5469175214816276E-2</v>
       </c>
       <c r="J57" s="10">
         <f t="shared" si="10"/>
-        <v>24582.780000000028</v>
+        <v>24576.589999999997</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
@@ -3311,10 +3311,10 @@
         <v>6</v>
       </c>
       <c r="D58" s="9">
-        <v>187631.67</v>
+        <v>187584.4</v>
       </c>
       <c r="E58" s="9">
-        <v>192370.76</v>
+        <v>192322.3</v>
       </c>
       <c r="F58" s="10" t="str">
         <f>IF(C58&lt;=fact_months,"",ROUND(D58*(1+Equalisation!$G$12/100)+IF(C58&gt;=equalisation_month,Equalisation!$F$12,0),2))</f>
@@ -3322,19 +3322,19 @@
       </c>
       <c r="G58" s="10">
         <f t="shared" si="6"/>
-        <v>192370.76</v>
+        <v>192322.3</v>
       </c>
       <c r="H58" s="10">
         <f t="shared" si="7"/>
-        <v>4739.0899999999965</v>
+        <v>4737.8999999999942</v>
       </c>
       <c r="I58" s="14">
         <f t="shared" si="8"/>
-        <v>2.5257409903136269E-2</v>
+        <v>2.5257430788487713E-2</v>
       </c>
       <c r="J58" s="10">
         <f t="shared" si="10"/>
-        <v>29321.870000000024</v>
+        <v>29314.489999999991</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
@@ -3348,10 +3348,10 @@
         <v>7</v>
       </c>
       <c r="D59" s="9">
-        <v>186468.66</v>
+        <v>186421.68</v>
       </c>
       <c r="E59" s="9">
-        <v>191099.95</v>
+        <v>191051.81</v>
       </c>
       <c r="F59" s="10" t="str">
         <f>IF(C59&lt;=fact_months,"",ROUND(D59*(1+Equalisation!$G$12/100)+IF(C59&gt;=equalisation_month,Equalisation!$F$12,0),2))</f>
@@ -3359,19 +3359,19 @@
       </c>
       <c r="G59" s="10">
         <f t="shared" si="6"/>
-        <v>191099.95</v>
+        <v>191051.81</v>
       </c>
       <c r="H59" s="10">
         <f t="shared" si="7"/>
-        <v>4631.2900000000081</v>
+        <v>4630.1300000000047</v>
       </c>
       <c r="I59" s="14">
         <f t="shared" si="8"/>
-        <v>2.4836827807954473E-2</v>
+        <v>2.4836864467694984E-2</v>
       </c>
       <c r="J59" s="10">
         <f t="shared" si="10"/>
-        <v>33953.160000000033</v>
+        <v>33944.619999999995</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.3">
@@ -3385,10 +3385,10 @@
         <v>8</v>
       </c>
       <c r="D60" s="9">
-        <v>186856.33</v>
+        <v>186809.26</v>
       </c>
       <c r="E60" s="9">
-        <v>191139.3</v>
+        <v>191091.16</v>
       </c>
       <c r="F60" s="10" t="str">
         <f>IF(C60&lt;=fact_months,"",ROUND(D60*(1+Equalisation!$G$12/100)+IF(C60&gt;=equalisation_month,Equalisation!$F$12,0),2))</f>
@@ -3396,19 +3396,19 @@
       </c>
       <c r="G60" s="10">
         <f t="shared" si="6"/>
-        <v>191139.3</v>
+        <v>191091.16</v>
       </c>
       <c r="H60" s="10">
         <f t="shared" si="7"/>
-        <v>4282.9700000000012</v>
+        <v>4281.8999999999942</v>
       </c>
       <c r="I60" s="14">
         <f t="shared" si="8"/>
-        <v>2.2921192982865508E-2</v>
+        <v>2.2921240628007381E-2</v>
       </c>
       <c r="J60" s="10">
         <f t="shared" si="10"/>
-        <v>38236.130000000034</v>
+        <v>38226.51999999999</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.3">
@@ -3422,28 +3422,28 @@
         <v>9</v>
       </c>
       <c r="D61" s="9">
-        <v>190926.85</v>
+        <v>190878.75</v>
       </c>
       <c r="E61" s="4"/>
       <c r="F61" s="10">
         <f>IF(C61&lt;=fact_months,"",ROUND(D61*(1+Equalisation!$G$12/100)+IF(C61&gt;=equalisation_month,Equalisation!$F$12,0),2))</f>
-        <v>195572.08</v>
+        <v>195522.81</v>
       </c>
       <c r="G61" s="10">
         <f t="shared" si="6"/>
-        <v>195572.08</v>
+        <v>195522.81</v>
       </c>
       <c r="H61" s="10">
         <f t="shared" si="7"/>
-        <v>4645.2299999999814</v>
+        <v>4644.0599999999977</v>
       </c>
       <c r="I61" s="14">
         <f t="shared" si="8"/>
-        <v>2.4329893883442696E-2</v>
+        <v>2.4329895286929519E-2</v>
       </c>
       <c r="J61" s="10">
         <f t="shared" si="10"/>
-        <v>42881.360000000015</v>
+        <v>42870.579999999987</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.3">
@@ -3457,28 +3457,28 @@
         <v>10</v>
       </c>
       <c r="D62" s="9">
-        <v>194997.37</v>
+        <v>194948.25</v>
       </c>
       <c r="E62" s="4"/>
       <c r="F62" s="10">
         <f>IF(C62&lt;=fact_months,"",ROUND(D62*(1+Equalisation!$G$12/100)+IF(C62&gt;=equalisation_month,Equalisation!$F$12,0),2))</f>
-        <v>199741.64</v>
+        <v>199691.32</v>
       </c>
       <c r="G62" s="10">
         <f t="shared" si="6"/>
-        <v>199741.64</v>
+        <v>199691.32</v>
       </c>
       <c r="H62" s="10">
         <f t="shared" si="7"/>
-        <v>4744.2700000000186</v>
+        <v>4743.070000000007</v>
       </c>
       <c r="I62" s="14">
         <f t="shared" si="8"/>
-        <v>2.4329917885559271E-2</v>
+        <v>2.4329892676646273E-2</v>
       </c>
       <c r="J62" s="10">
         <f t="shared" si="10"/>
-        <v>47625.630000000034</v>
+        <v>47613.649999999994</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.3">
@@ -3492,28 +3492,28 @@
         <v>11</v>
       </c>
       <c r="D63" s="9">
-        <v>196548.05</v>
+        <v>196498.53</v>
       </c>
       <c r="E63" s="4"/>
       <c r="F63" s="10">
         <f>IF(C63&lt;=fact_months,"",ROUND(D63*(1+Equalisation!$G$12/100)+IF(C63&gt;=equalisation_month,Equalisation!$F$12,0),2))</f>
-        <v>201330.05</v>
+        <v>201279.32</v>
       </c>
       <c r="G63" s="10">
         <f t="shared" si="6"/>
-        <v>201330.05</v>
+        <v>201279.32</v>
       </c>
       <c r="H63" s="10">
         <f t="shared" si="7"/>
-        <v>4782</v>
+        <v>4780.7900000000081</v>
       </c>
       <c r="I63" s="14">
         <f t="shared" si="8"/>
-        <v>2.4329928483136823E-2</v>
+        <v>2.432990211173594E-2</v>
       </c>
       <c r="J63" s="10">
         <f t="shared" si="10"/>
-        <v>52407.630000000034</v>
+        <v>52394.44</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
@@ -3527,28 +3527,28 @@
         <v>12</v>
       </c>
       <c r="D64" s="9">
-        <v>196741.88</v>
+        <v>196692.32</v>
       </c>
       <c r="E64" s="4"/>
       <c r="F64" s="10">
         <f>IF(C64&lt;=fact_months,"",ROUND(D64*(1+Equalisation!$G$12/100)+IF(C64&gt;=equalisation_month,Equalisation!$F$12,0),2))</f>
-        <v>201528.59</v>
+        <v>201477.83</v>
       </c>
       <c r="G64" s="10">
         <f t="shared" si="6"/>
-        <v>201528.59</v>
+        <v>201477.83</v>
       </c>
       <c r="H64" s="10">
         <f t="shared" si="7"/>
-        <v>4786.7099999999919</v>
+        <v>4785.5099999999802</v>
       </c>
       <c r="I64" s="14">
         <f t="shared" si="8"/>
-        <v>2.4329898646897101E-2</v>
+        <v>2.432992808260119E-2</v>
       </c>
       <c r="J64" s="10">
         <f t="shared" si="10"/>
-        <v>57194.340000000026</v>
+        <v>57179.949999999983</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
@@ -3998,10 +3998,10 @@
         <v>1</v>
       </c>
       <c r="D77" s="9">
-        <v>74139.31</v>
+        <v>74104.679999999993</v>
       </c>
       <c r="E77" s="9">
-        <v>76193.36</v>
+        <v>76157.77</v>
       </c>
       <c r="F77" s="10" t="str">
         <f>IF(C77&lt;=fact_months,"",ROUND(D77*(1+Equalisation!$G$14/100)+IF(C77&gt;=equalisation_month,Equalisation!$F$14,0),2))</f>
@@ -4009,19 +4009,19 @@
       </c>
       <c r="G77" s="10">
         <f t="shared" si="12"/>
-        <v>76193.36</v>
+        <v>76157.77</v>
       </c>
       <c r="H77" s="10">
         <f t="shared" si="13"/>
-        <v>2054.0500000000029</v>
+        <v>2053.0900000000111</v>
       </c>
       <c r="I77" s="14">
         <f t="shared" si="14"/>
-        <v>2.7705275379552398E-2</v>
+        <v>2.7705267737476381E-2</v>
       </c>
       <c r="J77" s="10">
         <f>H77</f>
-        <v>2054.0500000000029</v>
+        <v>2053.0900000000111</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.3">
@@ -4035,10 +4035,10 @@
         <v>2</v>
       </c>
       <c r="D78" s="9">
-        <v>73925.039999999994</v>
+        <v>73890.509999999995</v>
       </c>
       <c r="E78" s="9">
-        <v>75927.570000000007</v>
+        <v>75892.11</v>
       </c>
       <c r="F78" s="10" t="str">
         <f>IF(C78&lt;=fact_months,"",ROUND(D78*(1+Equalisation!$G$14/100)+IF(C78&gt;=equalisation_month,Equalisation!$F$14,0),2))</f>
@@ -4046,19 +4046,19 @@
       </c>
       <c r="G78" s="10">
         <f t="shared" si="12"/>
-        <v>75927.570000000007</v>
+        <v>75892.11</v>
       </c>
       <c r="H78" s="10">
         <f t="shared" si="13"/>
-        <v>2002.5300000000134</v>
+        <v>2001.6000000000058</v>
       </c>
       <c r="I78" s="14">
         <f t="shared" si="14"/>
-        <v>2.7088656292915278E-2</v>
+        <v>2.7088728985630306E-2</v>
       </c>
       <c r="J78" s="10">
         <f t="shared" ref="J78:J88" si="15">J77+H78</f>
-        <v>4056.5800000000163</v>
+        <v>4054.6900000000169</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.3">
@@ -4072,10 +4072,10 @@
         <v>3</v>
       </c>
       <c r="D79" s="9">
-        <v>72996.509999999995</v>
+        <v>72962.41</v>
       </c>
       <c r="E79" s="9">
-        <v>74921.460000000006</v>
+        <v>74886.460000000006</v>
       </c>
       <c r="F79" s="10" t="str">
         <f>IF(C79&lt;=fact_months,"",ROUND(D79*(1+Equalisation!$G$14/100)+IF(C79&gt;=equalisation_month,Equalisation!$F$14,0),2))</f>
@@ -4083,19 +4083,19 @@
       </c>
       <c r="G79" s="10">
         <f t="shared" si="12"/>
-        <v>74921.460000000006</v>
+        <v>74886.460000000006</v>
       </c>
       <c r="H79" s="10">
         <f t="shared" si="13"/>
-        <v>1924.9500000000116</v>
+        <v>1924.0500000000029</v>
       </c>
       <c r="I79" s="14">
         <f t="shared" si="14"/>
-        <v>2.6370438805910196E-2</v>
+        <v>2.6370428279438723E-2</v>
       </c>
       <c r="J79" s="10">
         <f t="shared" si="15"/>
-        <v>5981.5300000000279</v>
+        <v>5978.7400000000198</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.3">
@@ -4109,10 +4109,10 @@
         <v>4</v>
       </c>
       <c r="D80" s="9">
-        <v>71782.28</v>
+        <v>71748.75</v>
       </c>
       <c r="E80" s="9">
-        <v>73763.240000000005</v>
+        <v>73728.78</v>
       </c>
       <c r="F80" s="10" t="str">
         <f>IF(C80&lt;=fact_months,"",ROUND(D80*(1+Equalisation!$G$14/100)+IF(C80&gt;=equalisation_month,Equalisation!$F$14,0),2))</f>
@@ -4120,19 +4120,19 @@
       </c>
       <c r="G80" s="10">
         <f t="shared" si="12"/>
-        <v>73763.240000000005</v>
+        <v>73728.78</v>
       </c>
       <c r="H80" s="10">
         <f t="shared" si="13"/>
-        <v>1980.9600000000064</v>
+        <v>1980.0299999999988</v>
       </c>
       <c r="I80" s="14">
         <f t="shared" si="14"/>
-        <v>2.7596782938630625E-2</v>
+        <v>2.7596717712852124E-2</v>
       </c>
       <c r="J80" s="10">
         <f t="shared" si="15"/>
-        <v>7962.4900000000343</v>
+        <v>7958.7700000000186</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.3">
@@ -4146,10 +4146,10 @@
         <v>5</v>
       </c>
       <c r="D81" s="9">
-        <v>70425.2</v>
+        <v>70392.31</v>
       </c>
       <c r="E81" s="9">
-        <v>72393.899999999994</v>
+        <v>72360.09</v>
       </c>
       <c r="F81" s="10" t="str">
         <f>IF(C81&lt;=fact_months,"",ROUND(D81*(1+Equalisation!$G$14/100)+IF(C81&gt;=equalisation_month,Equalisation!$F$14,0),2))</f>
@@ -4157,19 +4157,19 @@
       </c>
       <c r="G81" s="10">
         <f t="shared" si="12"/>
-        <v>72393.899999999994</v>
+        <v>72360.09</v>
       </c>
       <c r="H81" s="10">
         <f t="shared" si="13"/>
-        <v>1968.6999999999971</v>
+        <v>1967.7799999999988</v>
       </c>
       <c r="I81" s="14">
         <f t="shared" si="14"/>
-        <v>2.7954482202393421E-2</v>
+        <v>2.7954474004333697E-2</v>
       </c>
       <c r="J81" s="10">
         <f t="shared" si="15"/>
-        <v>9931.1900000000314</v>
+        <v>9926.5500000000175</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.3">
@@ -4183,10 +4183,10 @@
         <v>6</v>
       </c>
       <c r="D82" s="9">
-        <v>69139.55</v>
+        <v>69107.259999999995</v>
       </c>
       <c r="E82" s="9">
-        <v>70937.710000000006</v>
+        <v>70904.58</v>
       </c>
       <c r="F82" s="10" t="str">
         <f>IF(C82&lt;=fact_months,"",ROUND(D82*(1+Equalisation!$G$14/100)+IF(C82&gt;=equalisation_month,Equalisation!$F$14,0),2))</f>
@@ -4194,19 +4194,19 @@
       </c>
       <c r="G82" s="10">
         <f t="shared" si="12"/>
-        <v>70937.710000000006</v>
+        <v>70904.58</v>
       </c>
       <c r="H82" s="10">
         <f t="shared" si="13"/>
-        <v>1798.1600000000035</v>
+        <v>1797.320000000007</v>
       </c>
       <c r="I82" s="14">
         <f t="shared" si="14"/>
-        <v>2.600769024386192E-2</v>
+        <v>2.6007687180768086E-2</v>
       </c>
       <c r="J82" s="10">
         <f t="shared" si="15"/>
-        <v>11729.350000000035</v>
+        <v>11723.870000000024</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.3">
@@ -4220,10 +4220,10 @@
         <v>7</v>
       </c>
       <c r="D83" s="9">
-        <v>68711</v>
+        <v>68678.91</v>
       </c>
       <c r="E83" s="9">
-        <v>70476.95</v>
+        <v>70444.039999999994</v>
       </c>
       <c r="F83" s="10" t="str">
         <f>IF(C83&lt;=fact_months,"",ROUND(D83*(1+Equalisation!$G$14/100)+IF(C83&gt;=equalisation_month,Equalisation!$F$14,0),2))</f>
@@ -4231,19 +4231,19 @@
       </c>
       <c r="G83" s="10">
         <f t="shared" si="12"/>
-        <v>70476.95</v>
+        <v>70444.039999999994</v>
       </c>
       <c r="H83" s="10">
         <f t="shared" si="13"/>
-        <v>1765.9499999999971</v>
+        <v>1765.1299999999901</v>
       </c>
       <c r="I83" s="14">
         <f t="shared" si="14"/>
-        <v>2.5701125001819172E-2</v>
+        <v>2.5701194151159214E-2</v>
       </c>
       <c r="J83" s="10">
         <f t="shared" si="15"/>
-        <v>13495.300000000032</v>
+        <v>13489.000000000015</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.3">
@@ -4257,10 +4257,10 @@
         <v>8</v>
       </c>
       <c r="D84" s="9">
-        <v>68853.850000000006</v>
+        <v>68821.69</v>
       </c>
       <c r="E84" s="9">
-        <v>70605.179999999993</v>
+        <v>70572.2</v>
       </c>
       <c r="F84" s="10" t="str">
         <f>IF(C84&lt;=fact_months,"",ROUND(D84*(1+Equalisation!$G$14/100)+IF(C84&gt;=equalisation_month,Equalisation!$F$14,0),2))</f>
@@ -4268,19 +4268,19 @@
       </c>
       <c r="G84" s="10">
         <f t="shared" si="12"/>
-        <v>70605.179999999993</v>
+        <v>70572.2</v>
       </c>
       <c r="H84" s="10">
         <f t="shared" si="13"/>
-        <v>1751.3299999999872</v>
+        <v>1750.5099999999948</v>
       </c>
       <c r="I84" s="14">
         <f t="shared" si="14"/>
-        <v>2.5435469476289083E-2</v>
+        <v>2.5435440483952004E-2</v>
       </c>
       <c r="J84" s="10">
         <f t="shared" si="15"/>
-        <v>15246.630000000019</v>
+        <v>15239.510000000009</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.3">
@@ -4294,28 +4294,28 @@
         <v>9</v>
       </c>
       <c r="D85" s="9">
-        <v>70353.78</v>
+        <v>70320.92</v>
       </c>
       <c r="E85" s="4"/>
       <c r="F85" s="10">
         <f>IF(C85&lt;=fact_months,"",ROUND(D85*(1+Equalisation!$G$14/100)+IF(C85&gt;=equalisation_month,Equalisation!$F$14,0),2))</f>
-        <v>73761.45</v>
+        <v>73724.820000000007</v>
       </c>
       <c r="G85" s="10">
         <f t="shared" si="12"/>
-        <v>73761.45</v>
+        <v>73724.820000000007</v>
       </c>
       <c r="H85" s="10">
         <f t="shared" si="13"/>
-        <v>3407.6699999999983</v>
+        <v>3403.9000000000087</v>
       </c>
       <c r="I85" s="14">
         <f t="shared" si="14"/>
-        <v>4.8436203427875496E-2</v>
+        <v>4.8405225642668054E-2</v>
       </c>
       <c r="J85" s="10">
         <f t="shared" si="15"/>
-        <v>18654.300000000017</v>
+        <v>18643.410000000018</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.3">
@@ -4329,28 +4329,28 @@
         <v>10</v>
       </c>
       <c r="D86" s="9">
-        <v>71853.710000000006</v>
+        <v>71820.149999999994</v>
       </c>
       <c r="E86" s="4"/>
       <c r="F86" s="10">
         <f>IF(C86&lt;=fact_months,"",ROUND(D86*(1+Equalisation!$G$14/100)+IF(C86&gt;=equalisation_month,Equalisation!$F$14,0),2))</f>
-        <v>75301.17</v>
+        <v>75263.820000000007</v>
       </c>
       <c r="G86" s="10">
         <f t="shared" si="12"/>
-        <v>75301.17</v>
+        <v>75263.820000000007</v>
       </c>
       <c r="H86" s="10">
         <f t="shared" si="13"/>
-        <v>3447.4599999999919</v>
+        <v>3443.6700000000128</v>
       </c>
       <c r="I86" s="14">
         <f t="shared" si="14"/>
-        <v>4.797887262884535E-2</v>
+        <v>4.7948521410774179E-2</v>
       </c>
       <c r="J86" s="10">
         <f t="shared" si="15"/>
-        <v>22101.760000000009</v>
+        <v>22087.080000000031</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.3">
@@ -4364,28 +4364,28 @@
         <v>11</v>
       </c>
       <c r="D87" s="9">
-        <v>72425.11</v>
+        <v>72391.28</v>
       </c>
       <c r="E87" s="4"/>
       <c r="F87" s="10">
         <f>IF(C87&lt;=fact_months,"",ROUND(D87*(1+Equalisation!$G$14/100)+IF(C87&gt;=equalisation_month,Equalisation!$F$14,0),2))</f>
-        <v>75887.72</v>
+        <v>75850.100000000006</v>
       </c>
       <c r="G87" s="10">
         <f t="shared" si="12"/>
-        <v>75887.72</v>
+        <v>75850.100000000006</v>
       </c>
       <c r="H87" s="10">
         <f t="shared" si="13"/>
-        <v>3462.6100000000006</v>
+        <v>3458.820000000007</v>
       </c>
       <c r="I87" s="14">
         <f t="shared" si="14"/>
-        <v>4.7809523520226625E-2</v>
+        <v>4.7779511565481464E-2</v>
       </c>
       <c r="J87" s="10">
         <f t="shared" si="15"/>
-        <v>25564.37000000001</v>
+        <v>25545.900000000038</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.3">
@@ -4399,28 +4399,28 @@
         <v>12</v>
       </c>
       <c r="D88" s="9">
-        <v>72496.53</v>
+        <v>72462.67</v>
       </c>
       <c r="E88" s="4"/>
       <c r="F88" s="10">
         <f>IF(C88&lt;=fact_months,"",ROUND(D88*(1+Equalisation!$G$14/100)+IF(C88&gt;=equalisation_month,Equalisation!$F$14,0),2))</f>
-        <v>75961.039999999994</v>
+        <v>75923.38</v>
       </c>
       <c r="G88" s="10">
         <f t="shared" si="12"/>
-        <v>75961.039999999994</v>
+        <v>75923.38</v>
       </c>
       <c r="H88" s="10">
         <f t="shared" si="13"/>
-        <v>3464.5099999999948</v>
+        <v>3460.7100000000064</v>
       </c>
       <c r="I88" s="14">
         <f t="shared" si="14"/>
-        <v>4.7788632090391012E-2</v>
+        <v>4.7758521732638427E-2</v>
       </c>
       <c r="J88" s="10">
         <f t="shared" si="15"/>
-        <v>29028.880000000005</v>
+        <v>29006.610000000044</v>
       </c>
     </row>
   </sheetData>
@@ -4499,23 +4499,23 @@
       </c>
       <c r="C6" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B6,Data!$D$5:$D$88)</f>
-        <v>1431549.17</v>
+        <v>1431233.43</v>
       </c>
       <c r="D6" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B6,Data!$G$5:$G$88)</f>
-        <v>1466464.76</v>
+        <v>1466137.25</v>
       </c>
       <c r="E6" s="10">
         <f t="shared" ref="E6:E17" si="0">D6-C6</f>
-        <v>34915.590000000084</v>
+        <v>34903.820000000065</v>
       </c>
       <c r="F6" s="14">
         <f t="shared" ref="F6:F18" si="1">E6/C6</f>
-        <v>2.4390073866621072E-2</v>
+        <v>2.438723080972198E-2</v>
       </c>
       <c r="G6" s="10">
         <f>E6</f>
-        <v>34915.590000000084</v>
+        <v>34903.820000000065</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -4527,23 +4527,23 @@
       </c>
       <c r="C7" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B7,Data!$D$5:$D$88)</f>
-        <v>1427411.7500000002</v>
+        <v>1427096.93</v>
       </c>
       <c r="D7" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B7,Data!$G$5:$G$88)</f>
-        <v>1462002.4000000001</v>
+        <v>1461675.87</v>
       </c>
       <c r="E7" s="10">
         <f t="shared" si="0"/>
-        <v>34590.649999999907</v>
+        <v>34578.940000000177</v>
       </c>
       <c r="F7" s="14">
         <f t="shared" si="1"/>
-        <v>2.4233126846545786E-2</v>
+        <v>2.4230267246107929E-2</v>
       </c>
       <c r="G7" s="10">
         <f t="shared" ref="G7:G17" si="2">G6+E7</f>
-        <v>69506.239999999991</v>
+        <v>69482.760000000242</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -4555,23 +4555,23 @@
       </c>
       <c r="C8" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B8,Data!$D$5:$D$88)</f>
-        <v>1409482.9100000001</v>
+        <v>1409172.02</v>
       </c>
       <c r="D8" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B8,Data!$G$5:$G$88)</f>
-        <v>1443777.85</v>
+        <v>1443455.41</v>
       </c>
       <c r="E8" s="10">
         <f t="shared" si="0"/>
-        <v>34294.939999999944</v>
+        <v>34283.389999999898</v>
       </c>
       <c r="F8" s="14">
         <f t="shared" si="1"/>
-        <v>2.4331575613073548E-2</v>
+        <v>2.4328747316456012E-2</v>
       </c>
       <c r="G8" s="10">
         <f t="shared" si="2"/>
-        <v>103801.17999999993</v>
+        <v>103766.15000000014</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -4583,23 +4583,23 @@
       </c>
       <c r="C9" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B9,Data!$D$5:$D$88)</f>
-        <v>1386037.4900000002</v>
+        <v>1385731.77</v>
       </c>
       <c r="D9" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B9,Data!$G$5:$G$88)</f>
-        <v>1420273.3900000001</v>
+        <v>1419956.1</v>
       </c>
       <c r="E9" s="10">
         <f t="shared" si="0"/>
-        <v>34235.899999999907</v>
+        <v>34224.330000000075</v>
       </c>
       <c r="F9" s="14">
         <f t="shared" si="1"/>
-        <v>2.4700558424289015E-2</v>
+        <v>2.4697658479750431E-2</v>
       </c>
       <c r="G9" s="10">
         <f t="shared" si="2"/>
-        <v>138037.07999999984</v>
+        <v>137990.48000000021</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -4611,23 +4611,23 @@
       </c>
       <c r="C10" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B10,Data!$D$5:$D$88)</f>
-        <v>1359833.7899999998</v>
+        <v>1359533.87</v>
       </c>
       <c r="D10" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B10,Data!$G$5:$G$88)</f>
-        <v>1393836.3399999999</v>
+        <v>1393524.95</v>
       </c>
       <c r="E10" s="10">
         <f t="shared" si="0"/>
-        <v>34002.550000000047</v>
+        <v>33991.079999999842</v>
       </c>
       <c r="F10" s="14">
         <f t="shared" si="1"/>
-        <v>2.5004930933507728E-2</v>
+        <v>2.5002010431707626E-2</v>
       </c>
       <c r="G10" s="10">
         <f t="shared" si="2"/>
-        <v>172039.62999999989</v>
+        <v>171981.56000000006</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -4639,23 +4639,23 @@
       </c>
       <c r="C11" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B11,Data!$D$5:$D$88)</f>
-        <v>1335009.25</v>
+        <v>1334714.79</v>
       </c>
       <c r="D11" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B11,Data!$G$5:$G$88)</f>
-        <v>1368196.2799999998</v>
+        <v>1367890.62</v>
       </c>
       <c r="E11" s="10">
         <f t="shared" si="0"/>
-        <v>33187.029999999795</v>
+        <v>33175.830000000075</v>
       </c>
       <c r="F11" s="14">
         <f t="shared" si="1"/>
-        <v>2.4859026257683079E-2</v>
+        <v>2.4856119261254365E-2</v>
       </c>
       <c r="G11" s="10">
         <f t="shared" si="2"/>
-        <v>205226.65999999968</v>
+        <v>205157.39000000013</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -4667,23 +4667,23 @@
       </c>
       <c r="C12" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B12,Data!$D$5:$D$88)</f>
-        <v>1326734.3899999999</v>
+        <v>1326441.7599999998</v>
       </c>
       <c r="D12" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B12,Data!$G$5:$G$88)</f>
-        <v>1358760.25</v>
+        <v>1358456.6700000002</v>
       </c>
       <c r="E12" s="10">
         <f t="shared" si="0"/>
-        <v>32025.860000000102</v>
+        <v>32014.910000000382</v>
       </c>
       <c r="F12" s="14">
         <f t="shared" si="1"/>
-        <v>2.4138863243003829E-2</v>
+        <v>2.4135933416330611E-2</v>
       </c>
       <c r="G12" s="10">
         <f t="shared" si="2"/>
-        <v>237252.51999999979</v>
+        <v>237172.30000000051</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -4695,23 +4695,23 @@
       </c>
       <c r="C13" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B13,Data!$D$5:$D$88)</f>
-        <v>1329492.6700000002</v>
+        <v>1329199.44</v>
       </c>
       <c r="D13" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B13,Data!$G$5:$G$88)</f>
-        <v>1362405.68</v>
+        <v>1362101.29</v>
       </c>
       <c r="E13" s="10">
         <f t="shared" si="0"/>
-        <v>32913.009999999776</v>
+        <v>32901.850000000093</v>
       </c>
       <c r="F13" s="14">
         <f t="shared" si="1"/>
-        <v>2.475606728993833E-2</v>
+        <v>2.4753132607398701E-2</v>
       </c>
       <c r="G13" s="10">
         <f t="shared" si="2"/>
-        <v>270165.52999999956</v>
+        <v>270074.15000000061</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -4723,23 +4723,23 @@
       </c>
       <c r="C14" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B14,Data!$D$5:$D$88)</f>
-        <v>1358454.6600000001</v>
+        <v>1358155.0299999998</v>
       </c>
       <c r="D14" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B14,Data!$G$5:$G$88)</f>
-        <v>1424841.45</v>
+        <v>1424507.42</v>
       </c>
       <c r="E14" s="10">
         <f t="shared" si="0"/>
-        <v>66386.789999999804</v>
+        <v>66352.39000000013</v>
       </c>
       <c r="F14" s="14">
         <f t="shared" si="1"/>
-        <v>4.8869345407523426E-2</v>
+        <v>4.8854798262610813E-2</v>
       </c>
       <c r="G14" s="10">
         <f t="shared" si="2"/>
-        <v>336552.31999999937</v>
+        <v>336426.54000000074</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -4751,23 +4751,23 @@
       </c>
       <c r="C15" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B15,Data!$D$5:$D$88)</f>
-        <v>1387416.65</v>
+        <v>1387110.63</v>
       </c>
       <c r="D15" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B15,Data!$G$5:$G$88)</f>
-        <v>1454514.3099999998</v>
+        <v>1454173.6600000001</v>
       </c>
       <c r="E15" s="10">
         <f t="shared" si="0"/>
-        <v>67097.659999999916</v>
+        <v>67063.030000000261</v>
       </c>
       <c r="F15" s="14">
         <f t="shared" si="1"/>
-        <v>4.8361579054136274E-2</v>
+        <v>4.8347282869572031E-2</v>
       </c>
       <c r="G15" s="10">
         <f t="shared" si="2"/>
-        <v>403649.97999999928</v>
+        <v>403489.570000001</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -4779,23 +4779,23 @@
       </c>
       <c r="C16" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B16,Data!$D$5:$D$88)</f>
-        <v>1398449.79</v>
+        <v>1398141.33</v>
       </c>
       <c r="D16" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B16,Data!$G$5:$G$88)</f>
-        <v>1465818.27</v>
+        <v>1465475.08</v>
       </c>
       <c r="E16" s="10">
         <f t="shared" si="0"/>
-        <v>67368.479999999981</v>
+        <v>67333.75</v>
       </c>
       <c r="F16" s="14">
         <f t="shared" si="1"/>
-        <v>4.8173685234705478E-2</v>
+        <v>4.8159473262978356E-2</v>
       </c>
       <c r="G16" s="10">
         <f t="shared" si="2"/>
-        <v>471018.45999999926</v>
+        <v>470823.320000001</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -4807,23 +4807,23 @@
       </c>
       <c r="C17" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B17,Data!$D$5:$D$88)</f>
-        <v>1399828.91</v>
+        <v>1399520.16</v>
       </c>
       <c r="D17" s="10">
         <f>SUMIF(Data!$C$5:$C$88,$B17,Data!$G$5:$G$88)</f>
-        <v>1467231.23</v>
+        <v>1466887.75</v>
       </c>
       <c r="E17" s="10">
         <f t="shared" si="0"/>
-        <v>67402.320000000065</v>
+        <v>67367.590000000084</v>
       </c>
       <c r="F17" s="14">
         <f t="shared" si="1"/>
-        <v>4.8150398608355696E-2</v>
+        <v>4.8136205483456623E-2</v>
       </c>
       <c r="G17" s="10">
         <f t="shared" si="2"/>
-        <v>538420.77999999933</v>
+        <v>538190.91000000108</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -4832,19 +4832,19 @@
       </c>
       <c r="C18" s="13">
         <f>SUM(C6:C17)</f>
-        <v>16549701.43</v>
+        <v>16546051.159999998</v>
       </c>
       <c r="D18" s="13">
         <f>SUM(D6:D17)</f>
-        <v>17088122.209999997</v>
+        <v>17084242.07</v>
       </c>
       <c r="E18" s="13">
         <f>SUM(E6:E17)</f>
-        <v>538420.77999999933</v>
+        <v>538190.91000000108</v>
       </c>
       <c r="F18" s="15">
         <f t="shared" si="1"/>
-        <v>3.2533564564735433E-2</v>
+        <v>3.2526849143382025E-2</v>
       </c>
     </row>
   </sheetData>
@@ -4916,39 +4916,39 @@
       </c>
       <c r="B5" s="10">
         <f>SUMIF(Data!$C$5:$C$16,"&lt;="&amp;fact_months,Data!$D$5:$D$16)</f>
-        <v>2651344.75</v>
+        <v>2650632.3000000003</v>
       </c>
       <c r="C5" s="10">
         <f>SUMIF(Data!$C$5:$C$16,"&lt;="&amp;fact_months,Data!$E$5:$E$16)</f>
-        <v>2612209.02</v>
+        <v>2611507.09</v>
       </c>
       <c r="D5" s="10">
         <f t="shared" ref="D5:D11" si="0">C5-B5</f>
-        <v>-39135.729999999981</v>
+        <v>-39125.210000000428</v>
       </c>
       <c r="E5" s="14">
         <f t="shared" ref="E5:E12" si="1">D5/B5</f>
-        <v>-1.4760709636119551E-2</v>
+        <v>-1.476070822799542E-2</v>
       </c>
       <c r="F5" s="10">
         <f>SUMIFS(Data!$F$5:$F$16,Data!$C$5:$C$16,"&gt;="&amp;equalisation_month)-SUMIFS(Data!$D$5:$D$16,Data!$C$5:$C$16,"&gt;="&amp;equalisation_month)</f>
-        <v>13426.850000000326</v>
+        <v>13423.260000000009</v>
       </c>
       <c r="G5" s="10">
         <f>SUM(Data!$D$5:$D$16)</f>
-        <v>3986984.5900000003</v>
+        <v>3985913.24</v>
       </c>
       <c r="H5" s="10">
         <f>SUM(Data!$G$5:$G$16)</f>
-        <v>3961275.71</v>
+        <v>3960211.29</v>
       </c>
       <c r="I5" s="10">
         <f t="shared" ref="I5:I11" si="2">H5-G5</f>
-        <v>-25708.880000000354</v>
+        <v>-25701.950000000186</v>
       </c>
       <c r="J5" s="14">
         <f t="shared" ref="J5:J12" si="3">I5/G5</f>
-        <v>-6.4482014965601738E-3</v>
+        <v>-6.4481960475387028E-3</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -4957,39 +4957,39 @@
       </c>
       <c r="B6" s="10">
         <f>SUMIF(Data!$C$17:$C$28,"&lt;="&amp;fact_months,Data!$D$17:$D$28)</f>
-        <v>1866910.9000000001</v>
+        <v>1866018.43</v>
       </c>
       <c r="C6" s="10">
         <f>SUMIF(Data!$C$17:$C$28,"&lt;="&amp;fact_months,Data!$E$17:$E$28)</f>
-        <v>2039420.2499999998</v>
+        <v>2038445.31</v>
       </c>
       <c r="D6" s="10">
         <f t="shared" si="0"/>
-        <v>172509.34999999963</v>
+        <v>172426.88000000012</v>
       </c>
       <c r="E6" s="14">
         <f t="shared" si="1"/>
-        <v>9.2403633188921669E-2</v>
+        <v>9.2403631833368402E-2</v>
       </c>
       <c r="F6" s="10">
         <f>SUMIFS(Data!$F$17:$F$28,Data!$C$17:$C$28,"&gt;="&amp;equalisation_month)-SUMIFS(Data!$D$17:$D$28,Data!$C$17:$C$28,"&gt;="&amp;equalisation_month)</f>
-        <v>130312.84000000008</v>
+        <v>130199.22999999975</v>
       </c>
       <c r="G6" s="10">
         <f>SUM(Data!$D$17:$D$28)</f>
-        <v>2807384.8200000008</v>
+        <v>2806042.75</v>
       </c>
       <c r="H6" s="10">
         <f>SUM(Data!$G$17:$G$28)</f>
-        <v>3110207.01</v>
+        <v>3108668.8600000003</v>
       </c>
       <c r="I6" s="10">
         <f t="shared" si="2"/>
-        <v>302822.18999999901</v>
+        <v>302626.11000000034</v>
       </c>
       <c r="J6" s="14">
         <f t="shared" si="3"/>
-        <v>0.10786629173267345</v>
+        <v>0.10784800409758559</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
@@ -4998,39 +4998,39 @@
       </c>
       <c r="B7" s="10">
         <f>SUMIF(Data!$C$29:$C$40,"&lt;="&amp;fact_months,Data!$D$29:$D$40)</f>
-        <v>1755011.6300000001</v>
+        <v>1754893.58</v>
       </c>
       <c r="C7" s="10">
         <f>SUMIF(Data!$C$29:$C$40,"&lt;="&amp;fact_months,Data!$E$29:$E$40)</f>
-        <v>1778274.8900000001</v>
+        <v>1778155.2899999998</v>
       </c>
       <c r="D7" s="10">
         <f t="shared" si="0"/>
-        <v>23263.260000000009</v>
+        <v>23261.70999999973</v>
       </c>
       <c r="E7" s="14">
         <f t="shared" si="1"/>
-        <v>1.325533096324838E-2</v>
+        <v>1.3255339392146919E-2</v>
       </c>
       <c r="F7" s="10">
         <f>SUMIFS(Data!$F$29:$F$40,Data!$C$29:$C$40,"&gt;="&amp;equalisation_month)-SUMIFS(Data!$D$29:$D$40,Data!$C$29:$C$40,"&gt;="&amp;equalisation_month)</f>
-        <v>18849.040000000037</v>
+        <v>18848.260000000009</v>
       </c>
       <c r="G7" s="10">
         <f>SUM(Data!$D$29:$D$40)</f>
-        <v>2639115.2400000002</v>
+        <v>2638937.7200000002</v>
       </c>
       <c r="H7" s="10">
         <f>SUM(Data!$G$29:$G$40)</f>
-        <v>2681227.54</v>
+        <v>2681047.69</v>
       </c>
       <c r="I7" s="10">
         <f t="shared" si="2"/>
-        <v>42112.299999999814</v>
+        <v>42109.969999999739</v>
       </c>
       <c r="J7" s="14">
         <f t="shared" si="3"/>
-        <v>1.5956976550974639E-2</v>
+        <v>1.5957167037651702E-2</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
@@ -5039,39 +5039,39 @@
       </c>
       <c r="B8" s="10">
         <f>SUMIF(Data!$C$41:$C$52,"&lt;="&amp;fact_months,Data!$D$41:$D$52)</f>
-        <v>1676619.77</v>
+        <v>1676571.22</v>
       </c>
       <c r="C8" s="10">
         <f>SUMIF(Data!$C$41:$C$52,"&lt;="&amp;fact_months,Data!$E$41:$E$52)</f>
-        <v>1716355.41</v>
+        <v>1716305.71</v>
       </c>
       <c r="D8" s="10">
         <f t="shared" si="0"/>
-        <v>39735.639999999898</v>
+        <v>39734.489999999991</v>
       </c>
       <c r="E8" s="14">
         <f t="shared" si="1"/>
-        <v>2.3699851755893286E-2</v>
+        <v>2.3699852130349697E-2</v>
       </c>
       <c r="F8" s="10">
         <f>SUMIFS(Data!$F$41:$F$52,Data!$C$41:$C$52,"&gt;="&amp;equalisation_month)-SUMIFS(Data!$D$41:$D$52,Data!$C$41:$C$52,"&gt;="&amp;equalisation_month)</f>
-        <v>48817.209999999846</v>
+        <v>48816.629999999888</v>
       </c>
       <c r="G8" s="10">
         <f>SUM(Data!$D$41:$D$52)</f>
-        <v>2521232.75</v>
+        <v>2521159.7199999997</v>
       </c>
       <c r="H8" s="10">
         <f>SUM(Data!$G$41:$G$52)</f>
-        <v>2609785.5999999996</v>
+        <v>2609710.84</v>
       </c>
       <c r="I8" s="10">
         <f t="shared" si="2"/>
-        <v>88552.849999999627</v>
+        <v>88551.120000000112</v>
       </c>
       <c r="J8" s="14">
         <f t="shared" si="3"/>
-        <v>3.5122838222690717E-2</v>
+        <v>3.5123169427758477E-2</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -5080,39 +5080,39 @@
       </c>
       <c r="B9" s="10">
         <f>SUMIF(Data!$C$53:$C$64,"&lt;="&amp;fact_months,Data!$D$53:$D$64)</f>
-        <v>1546798.25</v>
+        <v>1546408.5799999998</v>
       </c>
       <c r="C9" s="10">
         <f>SUMIF(Data!$C$53:$C$64,"&lt;="&amp;fact_months,Data!$E$53:$E$64)</f>
-        <v>1585034.38</v>
+        <v>1584635.1</v>
       </c>
       <c r="D9" s="10">
         <f t="shared" si="0"/>
-        <v>38236.129999999888</v>
+        <v>38226.520000000251</v>
       </c>
       <c r="E9" s="14">
         <f t="shared" si="1"/>
-        <v>2.4719532750958239E-2</v>
+        <v>2.4719547275145262E-2</v>
       </c>
       <c r="F9" s="10">
         <f>SUMIFS(Data!$F$53:$F$64,Data!$C$53:$C$64,"&gt;="&amp;equalisation_month)-SUMIFS(Data!$D$53:$D$64,Data!$C$53:$C$64,"&gt;="&amp;equalisation_month)</f>
-        <v>18958.209999999963</v>
+        <v>18953.429999999818</v>
       </c>
       <c r="G9" s="10">
         <f>SUM(Data!$D$53:$D$64)</f>
-        <v>2326012.4</v>
+        <v>2325426.4299999997</v>
       </c>
       <c r="H9" s="10">
         <f>SUM(Data!$G$53:$G$64)</f>
-        <v>2383206.7399999998</v>
+        <v>2382606.3800000004</v>
       </c>
       <c r="I9" s="10">
         <f t="shared" si="2"/>
-        <v>57194.339999999851</v>
+        <v>57179.950000000652</v>
       </c>
       <c r="J9" s="14">
         <f t="shared" si="3"/>
-        <v>2.4589009069771017E-2</v>
+        <v>2.458901699160642E-2</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
@@ -5162,39 +5162,39 @@
       </c>
       <c r="B11" s="10">
         <f>SUMIF(Data!$C$77:$C$88,"&lt;="&amp;fact_months,Data!$D$77:$D$88)</f>
-        <v>569972.74</v>
+        <v>569706.52</v>
       </c>
       <c r="C11" s="10">
         <f>SUMIF(Data!$C$77:$C$88,"&lt;="&amp;fact_months,Data!$E$77:$E$88)</f>
-        <v>585219.37000000011</v>
+        <v>584946.02999999991</v>
       </c>
       <c r="D11" s="10">
         <f t="shared" si="0"/>
-        <v>15246.630000000121</v>
+        <v>15239.509999999893</v>
       </c>
       <c r="E11" s="14">
         <f t="shared" si="1"/>
-        <v>2.6749752979414631E-2</v>
+        <v>2.6749755295059449E-2</v>
       </c>
       <c r="F11" s="10">
         <f>SUMIFS(Data!$F$77:$F$88,Data!$C$77:$C$88,"&gt;="&amp;equalisation_month)-SUMIFS(Data!$D$77:$D$88,Data!$C$77:$C$88,"&gt;="&amp;equalisation_month)</f>
-        <v>13782.25</v>
+        <v>13767.099999999977</v>
       </c>
       <c r="G11" s="10">
         <f>SUM(Data!$D$77:$D$88)</f>
-        <v>857101.87</v>
+        <v>856701.54000000015</v>
       </c>
       <c r="H11" s="10">
         <f>SUM(Data!$G$77:$G$88)</f>
-        <v>886130.75000000012</v>
+        <v>885708.14999999991</v>
       </c>
       <c r="I11" s="10">
         <f t="shared" si="2"/>
-        <v>29028.880000000121</v>
+        <v>29006.609999999753</v>
       </c>
       <c r="J11" s="14">
         <f t="shared" si="3"/>
-        <v>3.3868646208880776E-2</v>
+        <v>3.3858477714420528E-2</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
@@ -5203,39 +5203,39 @@
       </c>
       <c r="B12" s="13">
         <f>SUM(B5:B11)</f>
-        <v>11005551.42</v>
+        <v>11003124.009999998</v>
       </c>
       <c r="C12" s="13">
         <f>SUM(C5:C11)</f>
-        <v>11275716.949999999</v>
+        <v>11273198.16</v>
       </c>
       <c r="D12" s="13">
         <f>SUM(D5:D11)</f>
-        <v>270165.52999999968</v>
+        <v>270074.14999999967</v>
       </c>
       <c r="E12" s="15">
         <f t="shared" si="1"/>
-        <v>2.4548113919038841E-2</v>
+        <v>2.4545224588448468E-2</v>
       </c>
       <c r="F12" s="13">
         <f>SUM(F5:F11)</f>
-        <v>268255.25000000023</v>
+        <v>268116.75999999943</v>
       </c>
       <c r="G12" s="13">
         <f>SUM(G5:G11)</f>
-        <v>16549701.430000002</v>
+        <v>16546051.16</v>
       </c>
       <c r="H12" s="13">
         <f>SUM(H5:H11)</f>
-        <v>17088122.210000001</v>
+        <v>17084242.07</v>
       </c>
       <c r="I12" s="13">
         <f>SUM(I5:I11)</f>
-        <v>538420.7799999984</v>
+        <v>538190.91000000073</v>
       </c>
       <c r="J12" s="15">
         <f t="shared" si="3"/>
-        <v>3.2533564564735377E-2</v>
+        <v>3.2526849143381997E-2</v>
       </c>
     </row>
   </sheetData>
@@ -5298,7 +5298,7 @@
       </c>
       <c r="B5" s="10">
         <f>SUMIF(Monthly!$B$6:$B$17,"&lt;="&amp;fact_months,Monthly!$C$6:$C$17)</f>
-        <v>11005551.42</v>
+        <v>11003124.01</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>81</v>
@@ -5313,7 +5313,7 @@
       </c>
       <c r="B6" s="10">
         <f>SUMIF(Monthly!$B$6:$B$17,"&lt;="&amp;fact_months,Monthly!$D$6:$D$17)</f>
-        <v>11275716.949999999</v>
+        <v>11273198.16</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>84</v>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="B7" s="10">
         <f>B6-B5</f>
-        <v>270165.52999999933</v>
+        <v>270074.15000000037</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>87</v>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="B8" s="14">
         <f>B7/B5</f>
-        <v>2.454811391903881E-2</v>
+        <v>2.454522458844853E-2</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -5357,7 +5357,7 @@
       </c>
       <c r="B11" s="10">
         <f>Equalisation!$E$15</f>
-        <v>396521.56907576183</v>
+        <v>396244.5219988841</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -5366,7 +5366,7 @@
       </c>
       <c r="B12" s="10">
         <f>SUMIFS(Data!$F$5:$F$88,Data!$C$5:$C$88,"&gt;="&amp;equalisation_month)-SUMIFS(Data!$D$5:$D$88,Data!$C$5:$C$88,"&gt;="&amp;equalisation_month)</f>
-        <v>268255.24999999721</v>
+        <v>268116.75999999885</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="B15" s="10">
         <f>Monthly!$C$18</f>
-        <v>16549701.43</v>
+        <v>16546051.159999998</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -5389,7 +5389,7 @@
       </c>
       <c r="B16" s="10">
         <f>Monthly!$D$18</f>
-        <v>17088122.209999997</v>
+        <v>17084242.07</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -5398,7 +5398,7 @@
       </c>
       <c r="B17" s="10">
         <f>B16-B15</f>
-        <v>538420.77999999747</v>
+        <v>538190.91000000201</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="B18" s="14">
         <f>B17/B15</f>
-        <v>3.2533564564735322E-2</v>
+        <v>3.2526849143382081E-2</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -5566,7 +5566,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="91.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="103.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="18" t="s">
         <v>126</v>
       </c>

</xml_diff>